<commit_message>
docs(qa): mark 3228/3249/3250 tested; 3281 and Proposed Scope (3350-3367) ready for testing
- 3228, 3249, 3250: Tested = Yes / QA Status = Pass — tested and closed 15 Sept 2026
- 3281: QA Status = Ready for Testing — development complete
- Proposed Scope feature (DevOps 3350-3367, 18 items): added to the
  tracker as Dev Status = Done / QA Status = Ready for Testing.
  Confirmed implemented via code inspection (proposalField.js,
  links.js propagation/derivation logic, genModal.js/docxExport.js
  opt-in export) and a live browser smoke test (propose + filter).
  No formal QA test pass has been run yet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MRI_Taxonomy_Feature_List_QA_v2.0.xlsx
+++ b/MRI_Taxonomy_Feature_List_QA_v2.0.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1531" uniqueCount="592">
   <si>
     <t>MRI ERP Implementation Taxonomy — Feature List &amp; QA Tracker</t>
   </si>
@@ -1073,6 +1073,225 @@
   </si>
   <si>
     <t>Added from the 2026-09-14 board export, which raised this as a Feature. Built but had no tracker row and still has no user story beneath the feature.</t>
+  </si>
+  <si>
+    <t>Proposed Scope Tagging</t>
+  </si>
+  <si>
+    <t>Lets Open Box record, on either side of the taxonomy, where discovery has identified potential value add beyond what the client does today — a flag orthogonal to the existing coverage/scope tags, so the current-state tag is preserved.</t>
+  </si>
+  <si>
+    <t>src/components/proposalField.js, grid.js, businessView.js, genModal.js, docxExport.js; src/data/links.js</t>
+  </si>
+  <si>
+    <t>3350</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps Feature 3350. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Flag a value-stream process as Proposed Scope</t>
+  </si>
+  <si>
+    <t>A Propose control on each Value Streams card in Edit Mode; flagging it does not change the coverage tag; the card shows both tags together; saved with the version.</t>
+  </si>
+  <si>
+    <t>3352</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3352. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Flag an MRI PMX system process as Proposed Scope</t>
+  </si>
+  <si>
+    <t>A Propose control on each System view card in Edit Mode; the existing scope tag (Core/Custom/Out of scope) is retained; saved with the version.</t>
+  </si>
+  <si>
+    <t>3353</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3353. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Capture the value-add rationale for a proposal</t>
+  </si>
+  <si>
+    <t>Both edit modals expose a Proposed Scope checkbox and rationale field; the rationale appears in the detail panel and generated document; unticking clears it.</t>
+  </si>
+  <si>
+    <t>3354</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3354. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Distinguish a proposal from agreed client scope at a glance</t>
+  </si>
+  <si>
+    <t>Proposals use a distinct marker and dashed treatment, differing by shape as well as colour for colour-blind legibility; the panel states the item is a recommendation, not agreed scope.</t>
+  </si>
+  <si>
+    <t>3355</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3355. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Style the Proposed Scope tag to the Open Box brand palette</t>
+  </si>
+  <si>
+    <t>The ✦ PROPOSED chip and related badges use the Open Box brand colour (CSS var(--prop) / var(--prop-accent)).</t>
+  </si>
+  <si>
+    <t>3356</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3356. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Bulk-propose or clear proposals for a column</t>
+  </si>
+  <si>
+    <t>The Tag all menu in both views offers Propose all / Clear proposals, applied to every process and sub-process in the column, leaving coverage/scope tags untouched; one undo step.</t>
+  </si>
+  <si>
+    <t>3351</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3351. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Filter both views by Proposed Scope</t>
+  </si>
+  <si>
+    <t>A Proposed Scope toggle in both view filter bars narrows the existing coverage/scope selection rather than replacing it. Verified: toggling it hides non-proposed items and shows "No items match the selected filters" on empty columns.</t>
+  </si>
+  <si>
+    <t>3357</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3357. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Clear proposals when loading the Discovery Baseline</t>
+  </si>
+  <si>
+    <t>Loading the Discovery Baseline clears item proposals and proposed links on both sides, leaving the agreed link set intact (main.js clearProp / link filter on load).</t>
+  </si>
+  <si>
+    <t>3358</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3358. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Proposed Scope Propagation Across Links</t>
+  </si>
+  <si>
+    <t>Carries a proposal across existing business↔system links so it is only captured once; derivation is deliberately one-hop only to avoid cascading through the link graph.</t>
+  </si>
+  <si>
+    <t>3359</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps Feature 3359. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Imply a proposal across links in both directions</t>
+  </si>
+  <si>
+    <t>Flagging either side of a linked pair marks its linked counterparts as implied (derived); implied items render hollow/distinct from direct proposals, per links.js refreshDerivedProposals.</t>
+  </si>
+  <si>
+    <t>3360</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3360. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Prevent proposal propagation from cascading</t>
+  </si>
+  <si>
+    <t>Derivation reads only the directly-set `proposed` flag, never an implied one, so implication stops after one hop — confirmed in links.js comments and logic.</t>
+  </si>
+  <si>
+    <t>3361</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3361. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Propose a link that does not exist today</t>
+  </si>
+  <si>
+    <t>addLink() takes a `proposed` flag and toggleLinkProposed() exists; proposed links render dashed/distinct (map-chip-proposed, cell-flow-chip-proposed CSS).</t>
+  </si>
+  <si>
+    <t>3362</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3362. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Keep proposed links out of agreed-scope derivation</t>
+  </si>
+  <si>
+    <t>linkedSystemIds()/hasLink() filter out `proposed` links before deriving agreed scope (links.js), so a proposed link cannot lift an item out of auto out-of-scope.</t>
+  </si>
+  <si>
+    <t>3363</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3363. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Value-Add Proposals Document</t>
+  </si>
+  <si>
+    <t>Turns captured proposals into a client-facing section, excluded from generated documents unless explicitly included.</t>
+  </si>
+  <si>
+    <t>3364</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps Feature 3364. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Exclude proposals from generated documents by default</t>
+  </si>
+  <si>
+    <t>The export options include a Proposed Scope checkbox defaulting to unticked (genModal.js / docxExport.js inclProposed = false); no proposal content appears unless it is ticked.</t>
+  </si>
+  <si>
+    <t>3365</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3365. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Generate a Value-Add Proposals section</t>
+  </si>
+  <si>
+    <t>With Proposed Scope ticked, the document gains a Value-Add Proposals section grouped by side/module, opening with a recommendations-not-agreed-scope disclaimer (docxExport.js proposalsBlocks()).</t>
+  </si>
+  <si>
+    <t>3366</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3366. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+  </si>
+  <si>
+    <t>Nest linked counterparts under each proposal</t>
+  </si>
+  <si>
+    <t>Each proposal entry lists its linked counterparts as supporting detail, with proposed links marked as such in the list.</t>
+  </si>
+  <si>
+    <t>3367</t>
+  </si>
+  <si>
+    <t>Added 2026-10-01. DevOps User Story 3367. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
   </si>
   <si>
     <t>DevOps Backlog ⇄ App Feature Comparison</t>
@@ -1722,7 +1941,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1757,6 +1976,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF7F7F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD4EDDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -1860,7 +2084,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1937,6 +2161,9 @@
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
@@ -1946,7 +2173,7 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1994,10 +2221,10 @@
     <xf numFmtId="0" fontId="22" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2006,10 +2233,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2021,7 +2248,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2033,13 +2260,13 @@
     <xf numFmtId="9" fontId="28" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" indent="1"/>
     </xf>
-    <xf numFmtId="9" fontId="27" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="27" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2396,7 +2623,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K90"/>
+  <dimension ref="A1:K108"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -5486,6 +5713,636 @@
       </c>
       <c r="K90" s="25" t="s">
         <v>352</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A91" s="26">
+        <v>87</v>
+      </c>
+      <c r="B91" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="C91" s="26" t="s">
+        <v>353</v>
+      </c>
+      <c r="D91" s="26" t="s">
+        <v>354</v>
+      </c>
+      <c r="E91" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F91" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G91" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H91" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I91" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J91" s="26" t="s">
+        <v>356</v>
+      </c>
+      <c r="K91" s="26" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A92" s="26">
+        <v>88</v>
+      </c>
+      <c r="B92" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="C92" s="26" t="s">
+        <v>358</v>
+      </c>
+      <c r="D92" s="26" t="s">
+        <v>359</v>
+      </c>
+      <c r="E92" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F92" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G92" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H92" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I92" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J92" s="26" t="s">
+        <v>360</v>
+      </c>
+      <c r="K92" s="26" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A93" s="26">
+        <v>89</v>
+      </c>
+      <c r="B93" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="C93" s="26" t="s">
+        <v>362</v>
+      </c>
+      <c r="D93" s="26" t="s">
+        <v>363</v>
+      </c>
+      <c r="E93" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F93" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G93" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H93" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I93" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J93" s="26" t="s">
+        <v>364</v>
+      </c>
+      <c r="K93" s="26" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A94" s="26">
+        <v>90</v>
+      </c>
+      <c r="B94" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="C94" s="26" t="s">
+        <v>366</v>
+      </c>
+      <c r="D94" s="26" t="s">
+        <v>367</v>
+      </c>
+      <c r="E94" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F94" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G94" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H94" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I94" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J94" s="26" t="s">
+        <v>368</v>
+      </c>
+      <c r="K94" s="26" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A95" s="26">
+        <v>91</v>
+      </c>
+      <c r="B95" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="C95" s="26" t="s">
+        <v>370</v>
+      </c>
+      <c r="D95" s="26" t="s">
+        <v>371</v>
+      </c>
+      <c r="E95" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F95" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G95" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H95" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I95" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J95" s="26" t="s">
+        <v>372</v>
+      </c>
+      <c r="K95" s="26" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A96" s="26">
+        <v>92</v>
+      </c>
+      <c r="B96" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="C96" s="26" t="s">
+        <v>374</v>
+      </c>
+      <c r="D96" s="26" t="s">
+        <v>375</v>
+      </c>
+      <c r="E96" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F96" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G96" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H96" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I96" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J96" s="26" t="s">
+        <v>376</v>
+      </c>
+      <c r="K96" s="26" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A97" s="26">
+        <v>93</v>
+      </c>
+      <c r="B97" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="C97" s="26" t="s">
+        <v>378</v>
+      </c>
+      <c r="D97" s="26" t="s">
+        <v>379</v>
+      </c>
+      <c r="E97" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F97" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G97" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H97" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I97" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J97" s="26" t="s">
+        <v>380</v>
+      </c>
+      <c r="K97" s="26" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A98" s="26">
+        <v>94</v>
+      </c>
+      <c r="B98" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="C98" s="26" t="s">
+        <v>382</v>
+      </c>
+      <c r="D98" s="26" t="s">
+        <v>383</v>
+      </c>
+      <c r="E98" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F98" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G98" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H98" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I98" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J98" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="K98" s="26" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A99" s="26">
+        <v>95</v>
+      </c>
+      <c r="B99" s="26" t="s">
+        <v>186</v>
+      </c>
+      <c r="C99" s="26" t="s">
+        <v>386</v>
+      </c>
+      <c r="D99" s="26" t="s">
+        <v>387</v>
+      </c>
+      <c r="E99" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F99" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G99" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H99" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I99" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J99" s="26" t="s">
+        <v>388</v>
+      </c>
+      <c r="K99" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A100" s="26">
+        <v>96</v>
+      </c>
+      <c r="B100" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="C100" s="26" t="s">
+        <v>390</v>
+      </c>
+      <c r="D100" s="26" t="s">
+        <v>391</v>
+      </c>
+      <c r="E100" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F100" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G100" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H100" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I100" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J100" s="26" t="s">
+        <v>392</v>
+      </c>
+      <c r="K100" s="26" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A101" s="26">
+        <v>97</v>
+      </c>
+      <c r="B101" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="C101" s="26" t="s">
+        <v>394</v>
+      </c>
+      <c r="D101" s="26" t="s">
+        <v>395</v>
+      </c>
+      <c r="E101" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F101" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G101" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H101" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I101" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J101" s="26" t="s">
+        <v>396</v>
+      </c>
+      <c r="K101" s="26" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A102" s="26">
+        <v>98</v>
+      </c>
+      <c r="B102" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="C102" s="26" t="s">
+        <v>398</v>
+      </c>
+      <c r="D102" s="26" t="s">
+        <v>399</v>
+      </c>
+      <c r="E102" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F102" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G102" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H102" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I102" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J102" s="26" t="s">
+        <v>400</v>
+      </c>
+      <c r="K102" s="26" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A103" s="26">
+        <v>99</v>
+      </c>
+      <c r="B103" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="C103" s="26" t="s">
+        <v>402</v>
+      </c>
+      <c r="D103" s="26" t="s">
+        <v>403</v>
+      </c>
+      <c r="E103" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F103" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G103" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H103" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I103" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J103" s="26" t="s">
+        <v>404</v>
+      </c>
+      <c r="K103" s="26" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A104" s="26">
+        <v>100</v>
+      </c>
+      <c r="B104" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="C104" s="26" t="s">
+        <v>406</v>
+      </c>
+      <c r="D104" s="26" t="s">
+        <v>407</v>
+      </c>
+      <c r="E104" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F104" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G104" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H104" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I104" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J104" s="26" t="s">
+        <v>408</v>
+      </c>
+      <c r="K104" s="26" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A105" s="26">
+        <v>101</v>
+      </c>
+      <c r="B105" s="26" t="s">
+        <v>230</v>
+      </c>
+      <c r="C105" s="26" t="s">
+        <v>410</v>
+      </c>
+      <c r="D105" s="26" t="s">
+        <v>411</v>
+      </c>
+      <c r="E105" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F105" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G105" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H105" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I105" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J105" s="26" t="s">
+        <v>412</v>
+      </c>
+      <c r="K105" s="26" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A106" s="26">
+        <v>102</v>
+      </c>
+      <c r="B106" s="26" t="s">
+        <v>230</v>
+      </c>
+      <c r="C106" s="26" t="s">
+        <v>414</v>
+      </c>
+      <c r="D106" s="26" t="s">
+        <v>415</v>
+      </c>
+      <c r="E106" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F106" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G106" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H106" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I106" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J106" s="26" t="s">
+        <v>416</v>
+      </c>
+      <c r="K106" s="26" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A107" s="26">
+        <v>103</v>
+      </c>
+      <c r="B107" s="26" t="s">
+        <v>230</v>
+      </c>
+      <c r="C107" s="26" t="s">
+        <v>418</v>
+      </c>
+      <c r="D107" s="26" t="s">
+        <v>419</v>
+      </c>
+      <c r="E107" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F107" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G107" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H107" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I107" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J107" s="26" t="s">
+        <v>420</v>
+      </c>
+      <c r="K107" s="26" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A108" s="26">
+        <v>104</v>
+      </c>
+      <c r="B108" s="26" t="s">
+        <v>230</v>
+      </c>
+      <c r="C108" s="26" t="s">
+        <v>422</v>
+      </c>
+      <c r="D108" s="26" t="s">
+        <v>423</v>
+      </c>
+      <c r="E108" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="F108" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="G108" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H108" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I108" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="J108" s="26" t="s">
+        <v>424</v>
+      </c>
+      <c r="K108" s="26" t="s">
+        <v>425</v>
       </c>
     </row>
   </sheetData>
@@ -5541,1716 +6398,1716 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
-        <v>353</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
+      <c r="A1" s="27" t="s">
+        <v>426</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
     </row>
     <row r="2" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
-        <v>354</v>
-      </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
+      <c r="A2" s="28" t="s">
+        <v>427</v>
+      </c>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
-        <v>355</v>
-      </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
+      <c r="A3" s="29" t="s">
+        <v>428</v>
+      </c>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="29" t="s">
-        <v>356</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>357</v>
-      </c>
-      <c r="C4" s="29" t="s">
-        <v>358</v>
-      </c>
-      <c r="D4" s="29" t="s">
-        <v>359</v>
-      </c>
-      <c r="E4" s="29" t="s">
-        <v>360</v>
-      </c>
-      <c r="F4" s="29" t="s">
-        <v>361</v>
-      </c>
-      <c r="G4" s="29" t="s">
-        <v>362</v>
-      </c>
-      <c r="H4" s="29" t="s">
-        <v>363</v>
-      </c>
-      <c r="I4" s="29" t="s">
+      <c r="A4" s="30" t="s">
+        <v>429</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>430</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>431</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>432</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>433</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>434</v>
+      </c>
+      <c r="G4" s="30" t="s">
+        <v>435</v>
+      </c>
+      <c r="H4" s="30" t="s">
+        <v>436</v>
+      </c>
+      <c r="I4" s="30" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="30" t="s">
+      <c r="A5" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="31" t="s">
-        <v>364</v>
-      </c>
-      <c r="C5" s="32" t="s">
-        <v>365</v>
-      </c>
-      <c r="D5" s="33" t="s">
-        <v>366</v>
-      </c>
-      <c r="E5" s="32">
+      <c r="B5" s="32" t="s">
+        <v>437</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>438</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>439</v>
+      </c>
+      <c r="E5" s="33">
         <v>3</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="F5" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H5" s="31" t="s">
+      <c r="G5" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H5" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="35" t="s">
+      <c r="A6" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="36" t="s">
-        <v>368</v>
-      </c>
-      <c r="C6" s="37" t="s">
-        <v>365</v>
-      </c>
-      <c r="D6" s="38" t="s">
-        <v>369</v>
-      </c>
-      <c r="E6" s="37">
+      <c r="B6" s="37" t="s">
+        <v>441</v>
+      </c>
+      <c r="C6" s="38" t="s">
+        <v>438</v>
+      </c>
+      <c r="D6" s="39" t="s">
+        <v>442</v>
+      </c>
+      <c r="E6" s="38">
         <v>2</v>
       </c>
-      <c r="F6" s="36" t="s">
-        <v>370</v>
-      </c>
-      <c r="G6" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H6" s="36" t="s">
+      <c r="F6" s="37" t="s">
+        <v>443</v>
+      </c>
+      <c r="G6" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H6" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="30" t="s">
-        <v>371</v>
-      </c>
-      <c r="B7" s="31" t="s">
-        <v>372</v>
-      </c>
-      <c r="C7" s="32" t="s">
-        <v>365</v>
-      </c>
-      <c r="D7" s="33" t="s">
-        <v>366</v>
-      </c>
-      <c r="E7" s="32">
+      <c r="A7" s="31" t="s">
+        <v>444</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>445</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>438</v>
+      </c>
+      <c r="D7" s="34" t="s">
+        <v>439</v>
+      </c>
+      <c r="E7" s="33">
         <v>2</v>
       </c>
-      <c r="F7" s="31" t="s">
-        <v>373</v>
-      </c>
-      <c r="G7" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H7" s="31" t="s">
+      <c r="F7" s="32" t="s">
+        <v>446</v>
+      </c>
+      <c r="G7" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H7" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="35" t="s">
+      <c r="A8" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="36" t="s">
-        <v>374</v>
-      </c>
-      <c r="C8" s="37" t="s">
-        <v>375</v>
-      </c>
-      <c r="D8" s="38" t="s">
-        <v>376</v>
-      </c>
-      <c r="E8" s="37">
+      <c r="B8" s="37" t="s">
+        <v>447</v>
+      </c>
+      <c r="C8" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>449</v>
+      </c>
+      <c r="E8" s="38">
         <v>3</v>
       </c>
-      <c r="F8" s="36" t="s">
+      <c r="F8" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="G8" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H8" s="36" t="s">
+      <c r="G8" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H8" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="30" t="s">
+      <c r="A9" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="31" t="s">
-        <v>377</v>
-      </c>
-      <c r="C9" s="32" t="s">
-        <v>365</v>
-      </c>
-      <c r="D9" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="E9" s="32">
+      <c r="B9" s="32" t="s">
+        <v>450</v>
+      </c>
+      <c r="C9" s="33" t="s">
+        <v>438</v>
+      </c>
+      <c r="D9" s="34" t="s">
+        <v>442</v>
+      </c>
+      <c r="E9" s="33">
         <v>3</v>
       </c>
-      <c r="F9" s="31" t="s">
-        <v>378</v>
-      </c>
-      <c r="G9" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H9" s="31" t="s">
+      <c r="F9" s="32" t="s">
+        <v>451</v>
+      </c>
+      <c r="G9" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H9" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="35" t="s">
+      <c r="A10" s="36" t="s">
         <v>97</v>
       </c>
-      <c r="B10" s="36" t="s">
-        <v>379</v>
-      </c>
-      <c r="C10" s="37" t="s">
-        <v>375</v>
-      </c>
-      <c r="D10" s="38" t="s">
-        <v>380</v>
-      </c>
-      <c r="E10" s="37">
+      <c r="B10" s="37" t="s">
+        <v>452</v>
+      </c>
+      <c r="C10" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="D10" s="39" t="s">
+        <v>453</v>
+      </c>
+      <c r="E10" s="38">
         <v>2</v>
       </c>
-      <c r="F10" s="36" t="s">
+      <c r="F10" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="G10" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H10" s="36" t="s">
+      <c r="G10" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H10" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="B11" s="31" t="s">
-        <v>381</v>
-      </c>
-      <c r="C11" s="32" t="s">
-        <v>375</v>
-      </c>
-      <c r="D11" s="33" t="s">
-        <v>380</v>
-      </c>
-      <c r="E11" s="32">
+      <c r="B11" s="32" t="s">
+        <v>454</v>
+      </c>
+      <c r="C11" s="33" t="s">
+        <v>448</v>
+      </c>
+      <c r="D11" s="34" t="s">
+        <v>453</v>
+      </c>
+      <c r="E11" s="33">
         <v>3</v>
       </c>
-      <c r="F11" s="31" t="s">
+      <c r="F11" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="G11" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H11" s="31" t="s">
+      <c r="G11" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H11" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="35" t="s">
+      <c r="A12" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="B12" s="36" t="s">
-        <v>382</v>
-      </c>
-      <c r="C12" s="37" t="s">
-        <v>375</v>
-      </c>
-      <c r="D12" s="38" t="s">
-        <v>366</v>
-      </c>
-      <c r="E12" s="37">
+      <c r="B12" s="37" t="s">
+        <v>455</v>
+      </c>
+      <c r="C12" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="D12" s="39" t="s">
+        <v>439</v>
+      </c>
+      <c r="E12" s="38">
         <v>3</v>
       </c>
-      <c r="F12" s="36" t="s">
+      <c r="F12" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="G12" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H12" s="36" t="s">
+      <c r="G12" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H12" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="B13" s="31" t="s">
-        <v>383</v>
-      </c>
-      <c r="C13" s="32" t="s">
-        <v>384</v>
-      </c>
-      <c r="D13" s="33" t="s">
-        <v>366</v>
-      </c>
-      <c r="E13" s="32">
+      <c r="B13" s="32" t="s">
+        <v>456</v>
+      </c>
+      <c r="C13" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="D13" s="34" t="s">
+        <v>439</v>
+      </c>
+      <c r="E13" s="33">
         <v>2</v>
       </c>
-      <c r="F13" s="31" t="s">
+      <c r="F13" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="G13" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H13" s="31" t="s">
+      <c r="G13" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H13" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="35" t="s">
+      <c r="A14" s="36" t="s">
         <v>85</v>
       </c>
-      <c r="B14" s="36" t="s">
-        <v>385</v>
-      </c>
-      <c r="C14" s="37" t="s">
-        <v>375</v>
-      </c>
-      <c r="D14" s="38" t="s">
-        <v>366</v>
-      </c>
-      <c r="E14" s="37">
+      <c r="B14" s="37" t="s">
+        <v>458</v>
+      </c>
+      <c r="C14" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="D14" s="39" t="s">
+        <v>439</v>
+      </c>
+      <c r="E14" s="38">
         <v>2</v>
       </c>
-      <c r="F14" s="36" t="s">
+      <c r="F14" s="37" t="s">
         <v>82</v>
       </c>
-      <c r="G14" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H14" s="36" t="s">
+      <c r="G14" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H14" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="B15" s="31" t="s">
-        <v>386</v>
-      </c>
-      <c r="C15" s="32" t="s">
-        <v>375</v>
-      </c>
-      <c r="D15" s="33" t="s">
-        <v>366</v>
-      </c>
-      <c r="E15" s="32">
+      <c r="B15" s="32" t="s">
+        <v>459</v>
+      </c>
+      <c r="C15" s="33" t="s">
+        <v>448</v>
+      </c>
+      <c r="D15" s="34" t="s">
+        <v>439</v>
+      </c>
+      <c r="E15" s="33">
         <v>2</v>
       </c>
-      <c r="F15" s="31" t="s">
+      <c r="F15" s="32" t="s">
         <v>86</v>
       </c>
-      <c r="G15" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H15" s="31" t="s">
+      <c r="G15" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H15" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="35" t="s">
+      <c r="A16" s="36" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="36" t="s">
-        <v>387</v>
-      </c>
-      <c r="C16" s="37" t="s">
-        <v>365</v>
-      </c>
-      <c r="D16" s="38" t="s">
-        <v>369</v>
-      </c>
-      <c r="E16" s="37">
+      <c r="B16" s="37" t="s">
+        <v>460</v>
+      </c>
+      <c r="C16" s="38" t="s">
+        <v>438</v>
+      </c>
+      <c r="D16" s="39" t="s">
+        <v>442</v>
+      </c>
+      <c r="E16" s="38">
         <v>3</v>
       </c>
-      <c r="F16" s="36" t="s">
-        <v>388</v>
-      </c>
-      <c r="G16" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H16" s="36" t="s">
+      <c r="F16" s="37" t="s">
+        <v>461</v>
+      </c>
+      <c r="G16" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H16" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="30" t="s">
+      <c r="A17" s="31" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="31" t="s">
-        <v>389</v>
-      </c>
-      <c r="C17" s="32" t="s">
-        <v>365</v>
-      </c>
-      <c r="D17" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="E17" s="32">
+      <c r="B17" s="32" t="s">
+        <v>462</v>
+      </c>
+      <c r="C17" s="33" t="s">
+        <v>438</v>
+      </c>
+      <c r="D17" s="34" t="s">
+        <v>442</v>
+      </c>
+      <c r="E17" s="33">
         <v>3</v>
       </c>
-      <c r="F17" s="31" t="s">
-        <v>390</v>
-      </c>
-      <c r="G17" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H17" s="31" t="s">
+      <c r="F17" s="32" t="s">
+        <v>463</v>
+      </c>
+      <c r="G17" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H17" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="35" t="s">
+      <c r="A18" s="36" t="s">
         <v>174</v>
       </c>
-      <c r="B18" s="36" t="s">
-        <v>391</v>
-      </c>
-      <c r="C18" s="37" t="s">
-        <v>365</v>
-      </c>
-      <c r="D18" s="39" t="s">
-        <v>392</v>
-      </c>
-      <c r="E18" s="37">
+      <c r="B18" s="37" t="s">
+        <v>464</v>
+      </c>
+      <c r="C18" s="38" t="s">
+        <v>438</v>
+      </c>
+      <c r="D18" s="40" t="s">
+        <v>465</v>
+      </c>
+      <c r="E18" s="38">
         <v>3</v>
       </c>
-      <c r="F18" s="36" t="s">
+      <c r="F18" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="G18" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H18" s="36" t="s">
-        <v>393</v>
+      <c r="G18" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H18" s="37" t="s">
+        <v>466</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="30" t="s">
-        <v>394</v>
-      </c>
-      <c r="B19" s="31" t="s">
-        <v>395</v>
-      </c>
-      <c r="C19" s="32" t="s">
-        <v>365</v>
-      </c>
-      <c r="D19" s="40" t="s">
-        <v>392</v>
-      </c>
-      <c r="E19" s="32">
+      <c r="A19" s="31" t="s">
+        <v>467</v>
+      </c>
+      <c r="B19" s="32" t="s">
+        <v>468</v>
+      </c>
+      <c r="C19" s="33" t="s">
+        <v>438</v>
+      </c>
+      <c r="D19" s="41" t="s">
+        <v>465</v>
+      </c>
+      <c r="E19" s="33">
         <v>3</v>
       </c>
-      <c r="F19" s="31" t="s">
+      <c r="F19" s="32" t="s">
         <v>118</v>
       </c>
-      <c r="G19" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H19" s="31" t="s">
-        <v>393</v>
+      <c r="G19" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H19" s="32" t="s">
+        <v>466</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="35" t="s">
+      <c r="A20" s="36" t="s">
         <v>185</v>
       </c>
-      <c r="B20" s="36" t="s">
-        <v>396</v>
-      </c>
-      <c r="C20" s="37" t="s">
-        <v>365</v>
-      </c>
-      <c r="D20" s="41" t="s">
-        <v>392</v>
-      </c>
-      <c r="E20" s="37">
+      <c r="B20" s="37" t="s">
+        <v>469</v>
+      </c>
+      <c r="C20" s="38" t="s">
+        <v>438</v>
+      </c>
+      <c r="D20" s="42" t="s">
+        <v>465</v>
+      </c>
+      <c r="E20" s="38">
         <v>5</v>
       </c>
-      <c r="F20" s="36" t="s">
-        <v>397</v>
-      </c>
-      <c r="G20" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H20" s="36" t="s">
-        <v>393</v>
+      <c r="F20" s="37" t="s">
+        <v>470</v>
+      </c>
+      <c r="G20" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H20" s="37" t="s">
+        <v>466</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="30" t="s">
-        <v>398</v>
-      </c>
-      <c r="B21" s="31" t="s">
-        <v>399</v>
-      </c>
-      <c r="C21" s="32" t="s">
-        <v>365</v>
-      </c>
-      <c r="D21" s="42" t="s">
-        <v>392</v>
-      </c>
-      <c r="E21" s="32">
+      <c r="A21" s="31" t="s">
+        <v>471</v>
+      </c>
+      <c r="B21" s="32" t="s">
+        <v>472</v>
+      </c>
+      <c r="C21" s="33" t="s">
+        <v>438</v>
+      </c>
+      <c r="D21" s="43" t="s">
+        <v>465</v>
+      </c>
+      <c r="E21" s="33">
         <v>3</v>
       </c>
-      <c r="F21" s="31" t="s">
-        <v>400</v>
-      </c>
-      <c r="G21" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H21" s="31" t="s">
-        <v>393</v>
+      <c r="F21" s="32" t="s">
+        <v>473</v>
+      </c>
+      <c r="G21" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H21" s="32" t="s">
+        <v>466</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="35" t="s">
+      <c r="A22" s="36" t="s">
         <v>104</v>
       </c>
-      <c r="B22" s="36" t="s">
-        <v>401</v>
-      </c>
-      <c r="C22" s="37" t="s">
-        <v>375</v>
-      </c>
-      <c r="D22" s="38" t="s">
-        <v>369</v>
-      </c>
-      <c r="E22" s="37">
+      <c r="B22" s="37" t="s">
+        <v>474</v>
+      </c>
+      <c r="C22" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="D22" s="39" t="s">
+        <v>442</v>
+      </c>
+      <c r="E22" s="38">
         <v>5</v>
       </c>
-      <c r="F22" s="36" t="s">
-        <v>402</v>
-      </c>
-      <c r="G22" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H22" s="36" t="s">
+      <c r="F22" s="37" t="s">
+        <v>475</v>
+      </c>
+      <c r="G22" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H22" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="30" t="s">
+      <c r="A23" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="B23" s="31" t="s">
-        <v>403</v>
-      </c>
-      <c r="C23" s="32" t="s">
-        <v>375</v>
-      </c>
-      <c r="D23" s="33" t="s">
-        <v>392</v>
-      </c>
-      <c r="E23" s="32">
+      <c r="B23" s="32" t="s">
+        <v>476</v>
+      </c>
+      <c r="C23" s="33" t="s">
+        <v>448</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>465</v>
+      </c>
+      <c r="E23" s="33">
         <v>3</v>
       </c>
-      <c r="F23" s="31" t="s">
+      <c r="F23" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="G23" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H23" s="31" t="s">
+      <c r="G23" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H23" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="35" t="s">
+      <c r="A24" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="B24" s="36" t="s">
-        <v>404</v>
-      </c>
-      <c r="C24" s="37" t="s">
-        <v>375</v>
-      </c>
-      <c r="D24" s="38" t="s">
-        <v>369</v>
-      </c>
-      <c r="E24" s="37">
+      <c r="B24" s="37" t="s">
+        <v>477</v>
+      </c>
+      <c r="C24" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="D24" s="39" t="s">
+        <v>442</v>
+      </c>
+      <c r="E24" s="38">
         <v>3</v>
       </c>
-      <c r="F24" s="36" t="s">
+      <c r="F24" s="37" t="s">
         <v>105</v>
       </c>
-      <c r="G24" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H24" s="36" t="s">
+      <c r="G24" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H24" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="30" t="s">
-        <v>405</v>
-      </c>
-      <c r="B25" s="31" t="s">
-        <v>406</v>
-      </c>
-      <c r="C25" s="32" t="s">
-        <v>365</v>
-      </c>
-      <c r="D25" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="E25" s="32">
+      <c r="A25" s="31" t="s">
+        <v>478</v>
+      </c>
+      <c r="B25" s="32" t="s">
+        <v>479</v>
+      </c>
+      <c r="C25" s="33" t="s">
+        <v>438</v>
+      </c>
+      <c r="D25" s="34" t="s">
+        <v>442</v>
+      </c>
+      <c r="E25" s="33">
         <v>3</v>
       </c>
-      <c r="F25" s="31" t="s">
+      <c r="F25" s="32" t="s">
         <v>158</v>
       </c>
-      <c r="G25" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H25" s="31" t="s">
+      <c r="G25" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H25" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="35" t="s">
-        <v>407</v>
-      </c>
-      <c r="B26" s="36" t="s">
-        <v>408</v>
-      </c>
-      <c r="C26" s="37" t="s">
-        <v>375</v>
-      </c>
-      <c r="D26" s="38" t="s">
-        <v>409</v>
-      </c>
-      <c r="E26" s="37">
+      <c r="A26" s="36" t="s">
+        <v>480</v>
+      </c>
+      <c r="B26" s="37" t="s">
+        <v>481</v>
+      </c>
+      <c r="C26" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="D26" s="39" t="s">
+        <v>482</v>
+      </c>
+      <c r="E26" s="38">
         <v>2</v>
       </c>
-      <c r="F26" s="36" t="s">
-        <v>410</v>
-      </c>
-      <c r="G26" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H26" s="36" t="s">
-        <v>411</v>
+      <c r="F26" s="37" t="s">
+        <v>483</v>
+      </c>
+      <c r="G26" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H26" s="37" t="s">
+        <v>484</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="30" t="s">
+      <c r="A27" s="31" t="s">
         <v>165</v>
       </c>
-      <c r="B27" s="31" t="s">
-        <v>412</v>
-      </c>
-      <c r="C27" s="32" t="s">
-        <v>365</v>
-      </c>
-      <c r="D27" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="E27" s="32">
+      <c r="B27" s="32" t="s">
+        <v>485</v>
+      </c>
+      <c r="C27" s="33" t="s">
+        <v>438</v>
+      </c>
+      <c r="D27" s="34" t="s">
+        <v>442</v>
+      </c>
+      <c r="E27" s="33">
         <v>3</v>
       </c>
-      <c r="F27" s="31" t="s">
+      <c r="F27" s="32" t="s">
         <v>162</v>
       </c>
-      <c r="G27" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H27" s="31" t="s">
+      <c r="G27" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H27" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="35" t="s">
+      <c r="A28" s="36" t="s">
         <v>93</v>
       </c>
-      <c r="B28" s="36" t="s">
-        <v>413</v>
-      </c>
-      <c r="C28" s="37" t="s">
-        <v>375</v>
-      </c>
-      <c r="D28" s="38" t="s">
-        <v>369</v>
-      </c>
-      <c r="E28" s="37">
+      <c r="B28" s="37" t="s">
+        <v>486</v>
+      </c>
+      <c r="C28" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="D28" s="39" t="s">
+        <v>442</v>
+      </c>
+      <c r="E28" s="38">
         <v>3</v>
       </c>
-      <c r="F28" s="36" t="s">
+      <c r="F28" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="G28" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H28" s="36" t="s">
+      <c r="G28" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H28" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="30" t="s">
-        <v>414</v>
-      </c>
-      <c r="B29" s="31" t="s">
-        <v>415</v>
-      </c>
-      <c r="C29" s="32" t="s">
-        <v>384</v>
-      </c>
-      <c r="D29" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="E29" s="32">
+      <c r="A29" s="31" t="s">
+        <v>487</v>
+      </c>
+      <c r="B29" s="32" t="s">
+        <v>488</v>
+      </c>
+      <c r="C29" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="D29" s="34" t="s">
+        <v>442</v>
+      </c>
+      <c r="E29" s="33">
         <v>3</v>
       </c>
-      <c r="F29" s="31" t="s">
-        <v>416</v>
-      </c>
-      <c r="G29" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H29" s="31" t="s">
+      <c r="F29" s="32" t="s">
+        <v>489</v>
+      </c>
+      <c r="G29" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H29" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="35" t="s">
+      <c r="A30" s="36" t="s">
         <v>145</v>
       </c>
-      <c r="B30" s="36" t="s">
-        <v>417</v>
-      </c>
-      <c r="C30" s="37" t="s">
-        <v>375</v>
-      </c>
-      <c r="D30" s="38" t="s">
-        <v>366</v>
-      </c>
-      <c r="E30" s="37">
+      <c r="B30" s="37" t="s">
+        <v>490</v>
+      </c>
+      <c r="C30" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="D30" s="39" t="s">
+        <v>439</v>
+      </c>
+      <c r="E30" s="38">
         <v>3</v>
       </c>
-      <c r="F30" s="36" t="s">
+      <c r="F30" s="37" t="s">
         <v>142</v>
       </c>
-      <c r="G30" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H30" s="36" t="s">
+      <c r="G30" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H30" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="30" t="s">
+      <c r="A31" s="31" t="s">
         <v>157</v>
       </c>
-      <c r="B31" s="31" t="s">
-        <v>418</v>
-      </c>
-      <c r="C31" s="32" t="s">
-        <v>375</v>
-      </c>
-      <c r="D31" s="33" t="s">
-        <v>409</v>
-      </c>
-      <c r="E31" s="32">
+      <c r="B31" s="32" t="s">
+        <v>491</v>
+      </c>
+      <c r="C31" s="33" t="s">
+        <v>448</v>
+      </c>
+      <c r="D31" s="34" t="s">
+        <v>482</v>
+      </c>
+      <c r="E31" s="33">
         <v>5</v>
       </c>
-      <c r="F31" s="31" t="s">
+      <c r="F31" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="G31" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H31" s="31" t="s">
-        <v>419</v>
+      <c r="G31" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H31" s="32" t="s">
+        <v>492</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="35" t="s">
+      <c r="A32" s="36" t="s">
         <v>149</v>
       </c>
-      <c r="B32" s="36" t="s">
-        <v>420</v>
-      </c>
-      <c r="C32" s="37" t="s">
-        <v>384</v>
-      </c>
-      <c r="D32" s="38" t="s">
-        <v>369</v>
-      </c>
-      <c r="E32" s="37">
+      <c r="B32" s="37" t="s">
+        <v>493</v>
+      </c>
+      <c r="C32" s="38" t="s">
+        <v>457</v>
+      </c>
+      <c r="D32" s="39" t="s">
+        <v>442</v>
+      </c>
+      <c r="E32" s="38">
         <v>3</v>
       </c>
-      <c r="F32" s="36" t="s">
+      <c r="F32" s="37" t="s">
         <v>146</v>
       </c>
-      <c r="G32" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H32" s="36" t="s">
+      <c r="G32" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H32" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="30" t="s">
+      <c r="A33" s="31" t="s">
         <v>153</v>
       </c>
-      <c r="B33" s="31" t="s">
-        <v>421</v>
-      </c>
-      <c r="C33" s="32" t="s">
-        <v>375</v>
-      </c>
-      <c r="D33" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="E33" s="32">
+      <c r="B33" s="32" t="s">
+        <v>494</v>
+      </c>
+      <c r="C33" s="33" t="s">
+        <v>448</v>
+      </c>
+      <c r="D33" s="34" t="s">
+        <v>442</v>
+      </c>
+      <c r="E33" s="33">
         <v>3</v>
       </c>
-      <c r="F33" s="31" t="s">
+      <c r="F33" s="32" t="s">
         <v>150</v>
       </c>
-      <c r="G33" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H33" s="31" t="s">
+      <c r="G33" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H33" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="35" t="s">
-        <v>422</v>
-      </c>
-      <c r="B34" s="36" t="s">
-        <v>423</v>
-      </c>
-      <c r="C34" s="37" t="s">
-        <v>365</v>
-      </c>
-      <c r="D34" s="38" t="s">
-        <v>369</v>
-      </c>
-      <c r="E34" s="37">
+      <c r="A34" s="36" t="s">
+        <v>495</v>
+      </c>
+      <c r="B34" s="37" t="s">
+        <v>496</v>
+      </c>
+      <c r="C34" s="38" t="s">
+        <v>438</v>
+      </c>
+      <c r="D34" s="39" t="s">
+        <v>442</v>
+      </c>
+      <c r="E34" s="38">
         <v>5</v>
       </c>
-      <c r="F34" s="36" t="s">
-        <v>424</v>
-      </c>
-      <c r="G34" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H34" s="36" t="s">
+      <c r="F34" s="37" t="s">
+        <v>497</v>
+      </c>
+      <c r="G34" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H34" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="30" t="s">
-        <v>425</v>
-      </c>
-      <c r="B35" s="31" t="s">
-        <v>426</v>
-      </c>
-      <c r="C35" s="32" t="s">
-        <v>365</v>
-      </c>
-      <c r="D35" s="33" t="s">
-        <v>380</v>
-      </c>
-      <c r="E35" s="32">
+      <c r="A35" s="31" t="s">
+        <v>498</v>
+      </c>
+      <c r="B35" s="32" t="s">
+        <v>499</v>
+      </c>
+      <c r="C35" s="33" t="s">
+        <v>438</v>
+      </c>
+      <c r="D35" s="34" t="s">
+        <v>453</v>
+      </c>
+      <c r="E35" s="33">
         <v>5</v>
       </c>
-      <c r="F35" s="31" t="s">
-        <v>427</v>
-      </c>
-      <c r="G35" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H35" s="31" t="s">
+      <c r="F35" s="32" t="s">
+        <v>500</v>
+      </c>
+      <c r="G35" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H35" s="32" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="35" t="s">
+      <c r="A36" s="36" t="s">
         <v>262</v>
       </c>
-      <c r="B36" s="36" t="s">
-        <v>428</v>
-      </c>
-      <c r="C36" s="37" t="s">
-        <v>375</v>
-      </c>
-      <c r="D36" s="38" t="s">
-        <v>369</v>
-      </c>
-      <c r="E36" s="37">
+      <c r="B36" s="37" t="s">
+        <v>501</v>
+      </c>
+      <c r="C36" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="D36" s="39" t="s">
+        <v>442</v>
+      </c>
+      <c r="E36" s="38">
         <v>3</v>
       </c>
-      <c r="F36" s="36" t="s">
+      <c r="F36" s="37" t="s">
         <v>259</v>
       </c>
-      <c r="G36" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H36" s="36" t="s">
+      <c r="G36" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H36" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="30" t="s">
+      <c r="A37" s="31" t="s">
         <v>190</v>
       </c>
-      <c r="B37" s="31" t="s">
+      <c r="B37" s="32" t="s">
+        <v>502</v>
+      </c>
+      <c r="C37" s="33" t="s">
+        <v>438</v>
+      </c>
+      <c r="D37" s="34" t="s">
+        <v>442</v>
+      </c>
+      <c r="E37" s="33">
+        <v>5</v>
+      </c>
+      <c r="F37" s="32" t="s">
+        <v>503</v>
+      </c>
+      <c r="G37" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H37" s="32" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="36" t="s">
+        <v>194</v>
+      </c>
+      <c r="B38" s="37" t="s">
+        <v>504</v>
+      </c>
+      <c r="C38" s="38" t="s">
+        <v>438</v>
+      </c>
+      <c r="D38" s="39" t="s">
+        <v>465</v>
+      </c>
+      <c r="E38" s="38">
+        <v>3</v>
+      </c>
+      <c r="F38" s="37" t="s">
+        <v>191</v>
+      </c>
+      <c r="G38" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H38" s="37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="31" t="s">
+        <v>211</v>
+      </c>
+      <c r="B39" s="32" t="s">
+        <v>505</v>
+      </c>
+      <c r="C39" s="33" t="s">
+        <v>448</v>
+      </c>
+      <c r="D39" s="34" t="s">
+        <v>442</v>
+      </c>
+      <c r="E39" s="33">
+        <v>3</v>
+      </c>
+      <c r="F39" s="32" t="s">
+        <v>208</v>
+      </c>
+      <c r="G39" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H39" s="32" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="36" t="s">
+        <v>215</v>
+      </c>
+      <c r="B40" s="37" t="s">
+        <v>506</v>
+      </c>
+      <c r="C40" s="38" t="s">
+        <v>457</v>
+      </c>
+      <c r="D40" s="39" t="s">
+        <v>442</v>
+      </c>
+      <c r="E40" s="38">
+        <v>2</v>
+      </c>
+      <c r="F40" s="37" t="s">
+        <v>507</v>
+      </c>
+      <c r="G40" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H40" s="37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="31" t="s">
+        <v>223</v>
+      </c>
+      <c r="B41" s="32" t="s">
+        <v>508</v>
+      </c>
+      <c r="C41" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="D41" s="34" t="s">
+        <v>442</v>
+      </c>
+      <c r="E41" s="33">
+        <v>3</v>
+      </c>
+      <c r="F41" s="32" t="s">
+        <v>509</v>
+      </c>
+      <c r="G41" s="35" t="s">
+        <v>510</v>
+      </c>
+      <c r="H41" s="32" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="36" t="s">
+        <v>238</v>
+      </c>
+      <c r="B42" s="37" t="s">
+        <v>512</v>
+      </c>
+      <c r="C42" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="D42" s="39" t="s">
+        <v>442</v>
+      </c>
+      <c r="E42" s="38">
+        <v>5</v>
+      </c>
+      <c r="F42" s="37" t="s">
+        <v>513</v>
+      </c>
+      <c r="G42" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H42" s="37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="31" t="s">
+        <v>242</v>
+      </c>
+      <c r="B43" s="32" t="s">
+        <v>514</v>
+      </c>
+      <c r="C43" s="33" t="s">
+        <v>448</v>
+      </c>
+      <c r="D43" s="34" t="s">
+        <v>442</v>
+      </c>
+      <c r="E43" s="33">
+        <v>3</v>
+      </c>
+      <c r="F43" s="32" t="s">
+        <v>239</v>
+      </c>
+      <c r="G43" s="35" t="s">
+        <v>440</v>
+      </c>
+      <c r="H43" s="32" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="44" t="s">
+        <v>515</v>
+      </c>
+      <c r="B45" s="44"/>
+      <c r="C45" s="44"/>
+      <c r="D45" s="44"/>
+      <c r="E45" s="44"/>
+      <c r="F45" s="44"/>
+      <c r="G45" s="44"/>
+      <c r="H45" s="44"/>
+      <c r="I45" s="44"/>
+    </row>
+    <row r="46" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="30" t="s">
         <v>429</v>
       </c>
-      <c r="C37" s="32" t="s">
-        <v>365</v>
-      </c>
-      <c r="D37" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="E37" s="32">
+      <c r="B46" s="30" t="s">
+        <v>430</v>
+      </c>
+      <c r="C46" s="30" t="s">
+        <v>431</v>
+      </c>
+      <c r="D46" s="30" t="s">
+        <v>432</v>
+      </c>
+      <c r="E46" s="30" t="s">
+        <v>433</v>
+      </c>
+      <c r="F46" s="30" t="s">
+        <v>435</v>
+      </c>
+      <c r="G46" s="30" t="s">
+        <v>516</v>
+      </c>
+      <c r="H46" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="I46" s="30" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="31" t="s">
+        <v>269</v>
+      </c>
+      <c r="B47" s="32" t="s">
+        <v>265</v>
+      </c>
+      <c r="C47" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="D47" s="32" t="s">
+        <v>465</v>
+      </c>
+      <c r="E47" s="33">
+        <v>2</v>
+      </c>
+      <c r="F47" s="45" t="s">
+        <v>440</v>
+      </c>
+      <c r="G47" s="32" t="s">
+        <v>517</v>
+      </c>
+      <c r="H47" s="32"/>
+      <c r="I47" s="32"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="31" t="s">
+        <v>275</v>
+      </c>
+      <c r="B48" s="32" t="s">
+        <v>518</v>
+      </c>
+      <c r="C48" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="D48" s="32" t="s">
+        <v>482</v>
+      </c>
+      <c r="E48" s="33">
+        <v>2</v>
+      </c>
+      <c r="F48" s="46" t="s">
+        <v>519</v>
+      </c>
+      <c r="G48" s="32" t="s">
+        <v>520</v>
+      </c>
+      <c r="H48" s="32"/>
+      <c r="I48" s="32"/>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="31" t="s">
+        <v>282</v>
+      </c>
+      <c r="B49" s="32" t="s">
+        <v>278</v>
+      </c>
+      <c r="C49" s="33" t="s">
+        <v>521</v>
+      </c>
+      <c r="D49" s="32" t="s">
+        <v>482</v>
+      </c>
+      <c r="E49" s="33">
+        <v>8</v>
+      </c>
+      <c r="F49" s="46" t="s">
+        <v>519</v>
+      </c>
+      <c r="G49" s="32" t="s">
+        <v>522</v>
+      </c>
+      <c r="H49" s="32"/>
+      <c r="I49" s="32"/>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="31" t="s">
+        <v>286</v>
+      </c>
+      <c r="B50" s="32" t="s">
+        <v>523</v>
+      </c>
+      <c r="C50" s="33" t="s">
+        <v>521</v>
+      </c>
+      <c r="D50" s="32" t="s">
+        <v>482</v>
+      </c>
+      <c r="E50" s="33">
         <v>5</v>
       </c>
-      <c r="F37" s="31" t="s">
+      <c r="F50" s="46" t="s">
+        <v>519</v>
+      </c>
+      <c r="G50" s="32" t="s">
+        <v>524</v>
+      </c>
+      <c r="H50" s="32"/>
+      <c r="I50" s="32"/>
+    </row>
+    <row r="52" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="47" t="s">
+        <v>525</v>
+      </c>
+      <c r="B52" s="47"/>
+      <c r="C52" s="47"/>
+      <c r="D52" s="47"/>
+      <c r="E52" s="47"/>
+      <c r="F52" s="47"/>
+      <c r="G52" s="47"/>
+      <c r="H52" s="47"/>
+      <c r="I52" s="47"/>
+    </row>
+    <row r="53" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B53" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="C53" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D53" s="30" t="s">
+        <v>526</v>
+      </c>
+      <c r="E53" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="F53" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="G53" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H53" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="I53" s="30" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="48" t="s">
+        <v>23</v>
+      </c>
+      <c r="B54" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="C54" s="49" t="s">
+        <v>25</v>
+      </c>
+      <c r="D54" s="32" t="s">
+        <v>527</v>
+      </c>
+      <c r="E54" s="32"/>
+      <c r="F54" s="32"/>
+      <c r="G54" s="32"/>
+      <c r="H54" s="32"/>
+      <c r="I54" s="32"/>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="B55" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="C55" s="49" t="s">
+        <v>47</v>
+      </c>
+      <c r="D55" s="32" t="s">
+        <v>528</v>
+      </c>
+      <c r="E55" s="32"/>
+      <c r="F55" s="32"/>
+      <c r="G55" s="32"/>
+      <c r="H55" s="32"/>
+      <c r="I55" s="32"/>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" s="48" t="s">
+        <v>138</v>
+      </c>
+      <c r="B56" s="32" t="s">
+        <v>122</v>
+      </c>
+      <c r="C56" s="49" t="s">
+        <v>140</v>
+      </c>
+      <c r="D56" s="32" t="s">
+        <v>529</v>
+      </c>
+      <c r="E56" s="32"/>
+      <c r="F56" s="32"/>
+      <c r="G56" s="32"/>
+      <c r="H56" s="32"/>
+      <c r="I56" s="32"/>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" s="48" t="s">
+        <v>195</v>
+      </c>
+      <c r="B57" s="32" t="s">
+        <v>186</v>
+      </c>
+      <c r="C57" s="49" t="s">
+        <v>197</v>
+      </c>
+      <c r="D57" s="32" t="s">
+        <v>530</v>
+      </c>
+      <c r="E57" s="32"/>
+      <c r="F57" s="32"/>
+      <c r="G57" s="32"/>
+      <c r="H57" s="32"/>
+      <c r="I57" s="32"/>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" s="48" t="s">
+        <v>204</v>
+      </c>
+      <c r="B58" s="32" t="s">
+        <v>186</v>
+      </c>
+      <c r="C58" s="49" t="s">
+        <v>206</v>
+      </c>
+      <c r="D58" s="32" t="s">
+        <v>531</v>
+      </c>
+      <c r="E58" s="32"/>
+      <c r="F58" s="32"/>
+      <c r="G58" s="32"/>
+      <c r="H58" s="32"/>
+      <c r="I58" s="32"/>
+    </row>
+    <row r="60" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" s="50" t="s">
+        <v>532</v>
+      </c>
+      <c r="B60" s="50"/>
+      <c r="C60" s="50"/>
+      <c r="D60" s="50"/>
+      <c r="E60" s="50"/>
+      <c r="F60" s="50"/>
+      <c r="G60" s="50"/>
+      <c r="H60" s="50"/>
+      <c r="I60" s="50"/>
+    </row>
+    <row r="61" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A61" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B61" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="C61" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61" s="30" t="s">
+        <v>533</v>
+      </c>
+      <c r="E61" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="F61" s="30" t="s">
+        <v>534</v>
+      </c>
+      <c r="G61" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="H61" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="I61" s="30" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A62" s="48" t="s">
+        <v>288</v>
+      </c>
+      <c r="B62" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="C62" s="32" t="s">
+        <v>535</v>
+      </c>
+      <c r="D62" s="32" t="s">
+        <v>536</v>
+      </c>
+      <c r="E62" s="51" t="s">
+        <v>465</v>
+      </c>
+      <c r="F62" s="52" t="s">
+        <v>537</v>
+      </c>
+      <c r="G62" s="52"/>
+      <c r="H62" s="52"/>
+      <c r="I62" s="52"/>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63" s="48" t="s">
+        <v>293</v>
+      </c>
+      <c r="B63" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="C63" s="32" t="s">
+        <v>538</v>
+      </c>
+      <c r="D63" s="32" t="s">
+        <v>539</v>
+      </c>
+      <c r="E63" s="51" t="s">
+        <v>482</v>
+      </c>
+      <c r="F63" s="52" t="s">
+        <v>540</v>
+      </c>
+      <c r="G63" s="52"/>
+      <c r="H63" s="52"/>
+      <c r="I63" s="52"/>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64" s="48" t="s">
+        <v>296</v>
+      </c>
+      <c r="B64" s="32" t="s">
+        <v>141</v>
+      </c>
+      <c r="C64" s="32" t="s">
+        <v>541</v>
+      </c>
+      <c r="D64" s="32" t="s">
+        <v>542</v>
+      </c>
+      <c r="E64" s="51" t="s">
+        <v>482</v>
+      </c>
+      <c r="F64" s="52" t="s">
+        <v>543</v>
+      </c>
+      <c r="G64" s="52"/>
+      <c r="H64" s="52"/>
+      <c r="I64" s="52"/>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65" s="48" t="s">
+        <v>300</v>
+      </c>
+      <c r="B65" s="32" t="s">
+        <v>299</v>
+      </c>
+      <c r="C65" s="32" t="s">
+        <v>544</v>
+      </c>
+      <c r="D65" s="32" t="s">
+        <v>545</v>
+      </c>
+      <c r="E65" s="51" t="s">
+        <v>482</v>
+      </c>
+      <c r="F65" s="52" t="s">
+        <v>546</v>
+      </c>
+      <c r="G65" s="52"/>
+      <c r="H65" s="52"/>
+      <c r="I65" s="52"/>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" s="48" t="s">
+        <v>303</v>
+      </c>
+      <c r="B66" s="32" t="s">
+        <v>186</v>
+      </c>
+      <c r="C66" s="32" t="s">
+        <v>547</v>
+      </c>
+      <c r="D66" s="32" t="s">
+        <v>548</v>
+      </c>
+      <c r="E66" s="51" t="s">
+        <v>482</v>
+      </c>
+      <c r="F66" s="52" t="s">
+        <v>549</v>
+      </c>
+      <c r="G66" s="52"/>
+      <c r="H66" s="52"/>
+      <c r="I66" s="52"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" s="44" t="s">
+        <v>550</v>
+      </c>
+      <c r="B68" s="44"/>
+      <c r="C68" s="44"/>
+      <c r="D68" s="44"/>
+      <c r="E68" s="44"/>
+      <c r="F68" s="44"/>
+      <c r="G68" s="44"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" s="30" t="s">
+        <v>429</v>
+      </c>
+      <c r="B69" s="30" t="s">
         <v>430</v>
       </c>
-      <c r="G37" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H37" s="31" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="35" t="s">
-        <v>194</v>
-      </c>
-      <c r="B38" s="36" t="s">
+      <c r="C69" s="30" t="s">
         <v>431</v>
       </c>
-      <c r="C38" s="37" t="s">
-        <v>365</v>
-      </c>
-      <c r="D38" s="38" t="s">
-        <v>392</v>
-      </c>
-      <c r="E38" s="37">
+      <c r="D69" s="30" t="s">
+        <v>432</v>
+      </c>
+      <c r="E69" s="30" t="s">
+        <v>433</v>
+      </c>
+      <c r="F69" s="30" t="s">
+        <v>435</v>
+      </c>
+      <c r="G69" s="30" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" s="31" t="s">
+        <v>551</v>
+      </c>
+      <c r="B70" s="32" t="s">
+        <v>306</v>
+      </c>
+      <c r="C70" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="D70" s="32" t="s">
+        <v>482</v>
+      </c>
+      <c r="E70" s="33">
+        <v>8</v>
+      </c>
+      <c r="F70" s="45" t="s">
+        <v>519</v>
+      </c>
+      <c r="G70" s="32" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" s="31" t="s">
+        <v>553</v>
+      </c>
+      <c r="B71" s="32" t="s">
+        <v>311</v>
+      </c>
+      <c r="C71" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="D71" s="32" t="s">
+        <v>554</v>
+      </c>
+      <c r="E71" s="33">
+        <v>13</v>
+      </c>
+      <c r="F71" s="46" t="s">
+        <v>519</v>
+      </c>
+      <c r="G71" s="32" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" s="31" t="s">
+        <v>556</v>
+      </c>
+      <c r="B72" s="32" t="s">
+        <v>316</v>
+      </c>
+      <c r="C72" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="D72" s="32" t="s">
+        <v>465</v>
+      </c>
+      <c r="E72" s="33">
         <v>3</v>
       </c>
-      <c r="F38" s="36" t="s">
-        <v>191</v>
-      </c>
-      <c r="G38" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H38" s="36" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="30" t="s">
-        <v>211</v>
-      </c>
-      <c r="B39" s="31" t="s">
-        <v>432</v>
-      </c>
-      <c r="C39" s="32" t="s">
-        <v>375</v>
-      </c>
-      <c r="D39" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="E39" s="32">
-        <v>3</v>
-      </c>
-      <c r="F39" s="31" t="s">
-        <v>208</v>
-      </c>
-      <c r="G39" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H39" s="31" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="35" t="s">
-        <v>215</v>
-      </c>
-      <c r="B40" s="36" t="s">
-        <v>433</v>
-      </c>
-      <c r="C40" s="37" t="s">
-        <v>384</v>
-      </c>
-      <c r="D40" s="38" t="s">
-        <v>369</v>
-      </c>
-      <c r="E40" s="37">
-        <v>2</v>
-      </c>
-      <c r="F40" s="36" t="s">
-        <v>434</v>
-      </c>
-      <c r="G40" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H40" s="36" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="30" t="s">
-        <v>223</v>
-      </c>
-      <c r="B41" s="31" t="s">
-        <v>435</v>
-      </c>
-      <c r="C41" s="32" t="s">
-        <v>384</v>
-      </c>
-      <c r="D41" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="E41" s="32">
-        <v>3</v>
-      </c>
-      <c r="F41" s="31" t="s">
-        <v>436</v>
-      </c>
-      <c r="G41" s="34" t="s">
-        <v>437</v>
-      </c>
-      <c r="H41" s="31" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="35" t="s">
-        <v>238</v>
-      </c>
-      <c r="B42" s="36" t="s">
-        <v>439</v>
-      </c>
-      <c r="C42" s="37" t="s">
-        <v>375</v>
-      </c>
-      <c r="D42" s="38" t="s">
-        <v>369</v>
-      </c>
-      <c r="E42" s="37">
-        <v>5</v>
-      </c>
-      <c r="F42" s="36" t="s">
+      <c r="F72" s="45" t="s">
         <v>440</v>
       </c>
-      <c r="G42" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H42" s="36" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="30" t="s">
-        <v>242</v>
-      </c>
-      <c r="B43" s="31" t="s">
-        <v>441</v>
-      </c>
-      <c r="C43" s="32" t="s">
-        <v>375</v>
-      </c>
-      <c r="D43" s="33" t="s">
-        <v>369</v>
-      </c>
-      <c r="E43" s="32">
-        <v>3</v>
-      </c>
-      <c r="F43" s="31" t="s">
-        <v>239</v>
-      </c>
-      <c r="G43" s="34" t="s">
-        <v>367</v>
-      </c>
-      <c r="H43" s="31" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="43" t="s">
-        <v>442</v>
-      </c>
-      <c r="B45" s="43"/>
-      <c r="C45" s="43"/>
-      <c r="D45" s="43"/>
-      <c r="E45" s="43"/>
-      <c r="F45" s="43"/>
-      <c r="G45" s="43"/>
-      <c r="H45" s="43"/>
-      <c r="I45" s="43"/>
-    </row>
-    <row r="46" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="29" t="s">
-        <v>356</v>
-      </c>
-      <c r="B46" s="29" t="s">
-        <v>357</v>
-      </c>
-      <c r="C46" s="29" t="s">
-        <v>358</v>
-      </c>
-      <c r="D46" s="29" t="s">
-        <v>359</v>
-      </c>
-      <c r="E46" s="29" t="s">
-        <v>360</v>
-      </c>
-      <c r="F46" s="29" t="s">
-        <v>362</v>
-      </c>
-      <c r="G46" s="29" t="s">
-        <v>443</v>
-      </c>
-      <c r="H46" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="I46" s="29" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="30" t="s">
-        <v>269</v>
-      </c>
-      <c r="B47" s="31" t="s">
-        <v>265</v>
-      </c>
-      <c r="C47" s="32" t="s">
-        <v>384</v>
-      </c>
-      <c r="D47" s="31" t="s">
-        <v>392</v>
-      </c>
-      <c r="E47" s="32">
-        <v>2</v>
-      </c>
-      <c r="F47" s="44" t="s">
-        <v>367</v>
-      </c>
-      <c r="G47" s="31" t="s">
-        <v>444</v>
-      </c>
-      <c r="H47" s="31"/>
-      <c r="I47" s="31"/>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="30" t="s">
-        <v>275</v>
-      </c>
-      <c r="B48" s="31" t="s">
-        <v>445</v>
-      </c>
-      <c r="C48" s="32" t="s">
-        <v>384</v>
-      </c>
-      <c r="D48" s="31" t="s">
-        <v>409</v>
-      </c>
-      <c r="E48" s="32">
-        <v>2</v>
-      </c>
-      <c r="F48" s="45" t="s">
-        <v>446</v>
-      </c>
-      <c r="G48" s="31" t="s">
-        <v>447</v>
-      </c>
-      <c r="H48" s="31"/>
-      <c r="I48" s="31"/>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="30" t="s">
-        <v>282</v>
-      </c>
-      <c r="B49" s="31" t="s">
-        <v>278</v>
-      </c>
-      <c r="C49" s="32" t="s">
-        <v>448</v>
-      </c>
-      <c r="D49" s="31" t="s">
-        <v>409</v>
-      </c>
-      <c r="E49" s="32">
+      <c r="G72" s="32" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A73" s="31" t="s">
+        <v>558</v>
+      </c>
+      <c r="B73" s="32" t="s">
+        <v>320</v>
+      </c>
+      <c r="C73" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="D73" s="32" t="s">
+        <v>482</v>
+      </c>
+      <c r="E73" s="33">
         <v>8</v>
       </c>
-      <c r="F49" s="45" t="s">
-        <v>446</v>
-      </c>
-      <c r="G49" s="31" t="s">
-        <v>449</v>
-      </c>
-      <c r="H49" s="31"/>
-      <c r="I49" s="31"/>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="30" t="s">
-        <v>286</v>
-      </c>
-      <c r="B50" s="31" t="s">
-        <v>450</v>
-      </c>
-      <c r="C50" s="32" t="s">
-        <v>448</v>
-      </c>
-      <c r="D50" s="31" t="s">
-        <v>409</v>
-      </c>
-      <c r="E50" s="32">
-        <v>5</v>
-      </c>
-      <c r="F50" s="45" t="s">
-        <v>446</v>
-      </c>
-      <c r="G50" s="31" t="s">
-        <v>451</v>
-      </c>
-      <c r="H50" s="31"/>
-      <c r="I50" s="31"/>
-    </row>
-    <row r="52" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="46" t="s">
-        <v>452</v>
-      </c>
-      <c r="B52" s="46"/>
-      <c r="C52" s="46"/>
-      <c r="D52" s="46"/>
-      <c r="E52" s="46"/>
-      <c r="F52" s="46"/>
-      <c r="G52" s="46"/>
-      <c r="H52" s="46"/>
-      <c r="I52" s="46"/>
-    </row>
-    <row r="53" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" s="29" t="s">
-        <v>4</v>
-      </c>
-      <c r="B53" s="29" t="s">
-        <v>3</v>
-      </c>
-      <c r="C53" s="29" t="s">
-        <v>6</v>
-      </c>
-      <c r="D53" s="29" t="s">
-        <v>453</v>
-      </c>
-      <c r="E53" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="F53" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="G53" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="H53" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="I53" s="29" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A54" s="47" t="s">
-        <v>23</v>
-      </c>
-      <c r="B54" s="31" t="s">
-        <v>13</v>
-      </c>
-      <c r="C54" s="48" t="s">
-        <v>25</v>
-      </c>
-      <c r="D54" s="31" t="s">
-        <v>454</v>
-      </c>
-      <c r="E54" s="31"/>
-      <c r="F54" s="31"/>
-      <c r="G54" s="31"/>
-      <c r="H54" s="31"/>
-      <c r="I54" s="31"/>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="47" t="s">
-        <v>45</v>
-      </c>
-      <c r="B55" s="31" t="s">
-        <v>13</v>
-      </c>
-      <c r="C55" s="48" t="s">
-        <v>47</v>
-      </c>
-      <c r="D55" s="31" t="s">
-        <v>455</v>
-      </c>
-      <c r="E55" s="31"/>
-      <c r="F55" s="31"/>
-      <c r="G55" s="31"/>
-      <c r="H55" s="31"/>
-      <c r="I55" s="31"/>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A56" s="47" t="s">
-        <v>138</v>
-      </c>
-      <c r="B56" s="31" t="s">
-        <v>122</v>
-      </c>
-      <c r="C56" s="48" t="s">
-        <v>140</v>
-      </c>
-      <c r="D56" s="31" t="s">
-        <v>456</v>
-      </c>
-      <c r="E56" s="31"/>
-      <c r="F56" s="31"/>
-      <c r="G56" s="31"/>
-      <c r="H56" s="31"/>
-      <c r="I56" s="31"/>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A57" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="B57" s="31" t="s">
-        <v>186</v>
-      </c>
-      <c r="C57" s="48" t="s">
-        <v>197</v>
-      </c>
-      <c r="D57" s="31" t="s">
+      <c r="F73" s="46" t="s">
+        <v>510</v>
+      </c>
+      <c r="G73" s="32" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A74" s="31" t="s">
+        <v>560</v>
+      </c>
+      <c r="B74" s="32" t="s">
+        <v>324</v>
+      </c>
+      <c r="C74" s="33" t="s">
         <v>457</v>
       </c>
-      <c r="E57" s="31"/>
-      <c r="F57" s="31"/>
-      <c r="G57" s="31"/>
-      <c r="H57" s="31"/>
-      <c r="I57" s="31"/>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A58" s="47" t="s">
-        <v>204</v>
-      </c>
-      <c r="B58" s="31" t="s">
-        <v>186</v>
-      </c>
-      <c r="C58" s="48" t="s">
-        <v>206</v>
-      </c>
-      <c r="D58" s="31" t="s">
-        <v>458</v>
-      </c>
-      <c r="E58" s="31"/>
-      <c r="F58" s="31"/>
-      <c r="G58" s="31"/>
-      <c r="H58" s="31"/>
-      <c r="I58" s="31"/>
-    </row>
-    <row r="60" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A60" s="49" t="s">
-        <v>459</v>
-      </c>
-      <c r="B60" s="49"/>
-      <c r="C60" s="49"/>
-      <c r="D60" s="49"/>
-      <c r="E60" s="49"/>
-      <c r="F60" s="49"/>
-      <c r="G60" s="49"/>
-      <c r="H60" s="49"/>
-      <c r="I60" s="49"/>
-    </row>
-    <row r="61" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A61" s="29" t="s">
-        <v>4</v>
-      </c>
-      <c r="B61" s="29" t="s">
-        <v>3</v>
-      </c>
-      <c r="C61" s="29" t="s">
-        <v>5</v>
-      </c>
-      <c r="D61" s="29" t="s">
-        <v>460</v>
-      </c>
-      <c r="E61" s="29" t="s">
+      <c r="D74" s="32" t="s">
+        <v>482</v>
+      </c>
+      <c r="E74" s="33">
         <v>8</v>
       </c>
-      <c r="F61" s="29" t="s">
-        <v>461</v>
-      </c>
-      <c r="G61" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="H61" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="I61" s="29" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" s="47" t="s">
-        <v>288</v>
-      </c>
-      <c r="B62" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="C62" s="31" t="s">
-        <v>462</v>
-      </c>
-      <c r="D62" s="31" t="s">
-        <v>463</v>
-      </c>
-      <c r="E62" s="50" t="s">
-        <v>392</v>
-      </c>
-      <c r="F62" s="51" t="s">
-        <v>464</v>
-      </c>
-      <c r="G62" s="51"/>
-      <c r="H62" s="51"/>
-      <c r="I62" s="51"/>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A63" s="47" t="s">
-        <v>293</v>
-      </c>
-      <c r="B63" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="C63" s="31" t="s">
-        <v>465</v>
-      </c>
-      <c r="D63" s="31" t="s">
-        <v>466</v>
-      </c>
-      <c r="E63" s="50" t="s">
-        <v>409</v>
-      </c>
-      <c r="F63" s="51" t="s">
-        <v>467</v>
-      </c>
-      <c r="G63" s="51"/>
-      <c r="H63" s="51"/>
-      <c r="I63" s="51"/>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A64" s="47" t="s">
-        <v>296</v>
-      </c>
-      <c r="B64" s="31" t="s">
-        <v>141</v>
-      </c>
-      <c r="C64" s="31" t="s">
-        <v>468</v>
-      </c>
-      <c r="D64" s="31" t="s">
-        <v>469</v>
-      </c>
-      <c r="E64" s="50" t="s">
-        <v>409</v>
-      </c>
-      <c r="F64" s="51" t="s">
-        <v>470</v>
-      </c>
-      <c r="G64" s="51"/>
-      <c r="H64" s="51"/>
-      <c r="I64" s="51"/>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A65" s="47" t="s">
-        <v>300</v>
-      </c>
-      <c r="B65" s="31" t="s">
-        <v>299</v>
-      </c>
-      <c r="C65" s="31" t="s">
-        <v>471</v>
-      </c>
-      <c r="D65" s="31" t="s">
-        <v>472</v>
-      </c>
-      <c r="E65" s="50" t="s">
-        <v>409</v>
-      </c>
-      <c r="F65" s="51" t="s">
-        <v>473</v>
-      </c>
-      <c r="G65" s="51"/>
-      <c r="H65" s="51"/>
-      <c r="I65" s="51"/>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A66" s="47" t="s">
-        <v>303</v>
-      </c>
-      <c r="B66" s="31" t="s">
-        <v>186</v>
-      </c>
-      <c r="C66" s="31" t="s">
-        <v>474</v>
-      </c>
-      <c r="D66" s="31" t="s">
-        <v>475</v>
-      </c>
-      <c r="E66" s="50" t="s">
-        <v>409</v>
-      </c>
-      <c r="F66" s="51" t="s">
-        <v>476</v>
-      </c>
-      <c r="G66" s="51"/>
-      <c r="H66" s="51"/>
-      <c r="I66" s="51"/>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="43" t="s">
-        <v>477</v>
-      </c>
-      <c r="B68" s="43"/>
-      <c r="C68" s="43"/>
-      <c r="D68" s="43"/>
-      <c r="E68" s="43"/>
-      <c r="F68" s="43"/>
-      <c r="G68" s="43"/>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" s="29" t="s">
-        <v>356</v>
-      </c>
-      <c r="B69" s="29" t="s">
-        <v>357</v>
-      </c>
-      <c r="C69" s="29" t="s">
-        <v>358</v>
-      </c>
-      <c r="D69" s="29" t="s">
-        <v>359</v>
-      </c>
-      <c r="E69" s="29" t="s">
-        <v>360</v>
-      </c>
-      <c r="F69" s="29" t="s">
-        <v>362</v>
-      </c>
-      <c r="G69" s="29" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" s="30" t="s">
-        <v>478</v>
-      </c>
-      <c r="B70" s="31" t="s">
-        <v>306</v>
-      </c>
-      <c r="C70" s="32" t="s">
-        <v>384</v>
-      </c>
-      <c r="D70" s="31" t="s">
-        <v>409</v>
-      </c>
-      <c r="E70" s="32">
+      <c r="F74" s="45" t="s">
+        <v>519</v>
+      </c>
+      <c r="G74" s="32" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A75" s="31" t="s">
+        <v>562</v>
+      </c>
+      <c r="B75" s="32" t="s">
+        <v>327</v>
+      </c>
+      <c r="C75" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="D75" s="32" t="s">
+        <v>482</v>
+      </c>
+      <c r="E75" s="33">
         <v>8</v>
       </c>
-      <c r="F70" s="44" t="s">
-        <v>446</v>
-      </c>
-      <c r="G70" s="31" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="30" t="s">
-        <v>480</v>
-      </c>
-      <c r="B71" s="31" t="s">
-        <v>311</v>
-      </c>
-      <c r="C71" s="32" t="s">
-        <v>384</v>
-      </c>
-      <c r="D71" s="31" t="s">
-        <v>481</v>
-      </c>
-      <c r="E71" s="32">
-        <v>13</v>
-      </c>
-      <c r="F71" s="45" t="s">
-        <v>446</v>
-      </c>
-      <c r="G71" s="31" t="s">
+      <c r="F75" s="46" t="s">
+        <v>519</v>
+      </c>
+      <c r="G75" s="32" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76" s="31" t="s">
+        <v>332</v>
+      </c>
+      <c r="B76" s="32" t="s">
+        <v>330</v>
+      </c>
+      <c r="C76" s="33" t="s">
+        <v>457</v>
+      </c>
+      <c r="D76" s="32" t="s">
         <v>482</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" s="30" t="s">
-        <v>483</v>
-      </c>
-      <c r="B72" s="31" t="s">
-        <v>316</v>
-      </c>
-      <c r="C72" s="32" t="s">
-        <v>384</v>
-      </c>
-      <c r="D72" s="31" t="s">
-        <v>392</v>
-      </c>
-      <c r="E72" s="32">
-        <v>3</v>
-      </c>
-      <c r="F72" s="44" t="s">
-        <v>367</v>
-      </c>
-      <c r="G72" s="31" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" s="30" t="s">
-        <v>485</v>
-      </c>
-      <c r="B73" s="31" t="s">
-        <v>320</v>
-      </c>
-      <c r="C73" s="32" t="s">
-        <v>384</v>
-      </c>
-      <c r="D73" s="31" t="s">
-        <v>409</v>
-      </c>
-      <c r="E73" s="32">
-        <v>8</v>
-      </c>
-      <c r="F73" s="45" t="s">
-        <v>437</v>
-      </c>
-      <c r="G73" s="31" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A74" s="30" t="s">
-        <v>487</v>
-      </c>
-      <c r="B74" s="31" t="s">
-        <v>324</v>
-      </c>
-      <c r="C74" s="32" t="s">
-        <v>384</v>
-      </c>
-      <c r="D74" s="31" t="s">
-        <v>409</v>
-      </c>
-      <c r="E74" s="32">
-        <v>8</v>
-      </c>
-      <c r="F74" s="44" t="s">
-        <v>446</v>
-      </c>
-      <c r="G74" s="31" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="30" t="s">
-        <v>489</v>
-      </c>
-      <c r="B75" s="31" t="s">
-        <v>327</v>
-      </c>
-      <c r="C75" s="32" t="s">
-        <v>384</v>
-      </c>
-      <c r="D75" s="31" t="s">
-        <v>409</v>
-      </c>
-      <c r="E75" s="32">
-        <v>8</v>
-      </c>
-      <c r="F75" s="45" t="s">
-        <v>446</v>
-      </c>
-      <c r="G75" s="31" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" s="30" t="s">
-        <v>332</v>
-      </c>
-      <c r="B76" s="31" t="s">
-        <v>330</v>
-      </c>
-      <c r="C76" s="32" t="s">
-        <v>384</v>
-      </c>
-      <c r="D76" s="31" t="s">
-        <v>409</v>
-      </c>
-      <c r="E76" s="32" t="s">
-        <v>491</v>
-      </c>
-      <c r="F76" s="44" t="s">
-        <v>446</v>
-      </c>
-      <c r="G76" s="31" t="s">
-        <v>492</v>
+      <c r="E76" s="33" t="s">
+        <v>564</v>
+      </c>
+      <c r="F76" s="45" t="s">
+        <v>519</v>
+      </c>
+      <c r="G76" s="32" t="s">
+        <v>565</v>
       </c>
     </row>
   </sheetData>
@@ -7292,305 +8149,305 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="52" t="s">
-        <v>493</v>
-      </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
+      <c r="A1" s="53" t="s">
+        <v>566</v>
+      </c>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="53" t="s">
-        <v>494</v>
-      </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
+      <c r="A3" s="54" t="s">
+        <v>567</v>
+      </c>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="54" t="s">
-        <v>495</v>
-      </c>
-      <c r="C4" s="54" t="s">
-        <v>496</v>
+      <c r="B4" s="55" t="s">
+        <v>568</v>
+      </c>
+      <c r="C4" s="55" t="s">
+        <v>569</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="56">
+      <c r="A5" s="56" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="57">
         <f>COUNTIF('Feature List'!$G$5:$G$200,"Done")</f>
       </c>
-      <c r="C5" s="57">
+      <c r="C5" s="58">
         <f>IF(COUNTA('Feature List'!$G$5:$G$200)=0,0,COUNTIF('Feature List'!$G$5:$G$200,"Done")/COUNTA('Feature List'!$G$5:$G$200))</f>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="55" t="s">
+      <c r="A6" s="56" t="s">
         <v>314</v>
       </c>
-      <c r="B6" s="56">
+      <c r="B6" s="57">
         <f>COUNTIF('Feature List'!$G$5:$G$200,"In Progress")</f>
       </c>
-      <c r="C6" s="57">
+      <c r="C6" s="58">
         <f>IF(COUNTA('Feature List'!$G$5:$G$200)=0,0,COUNTIF('Feature List'!$G$5:$G$200,"In Progress")/COUNTA('Feature List'!$G$5:$G$200))</f>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="55" t="s">
+      <c r="A7" s="56" t="s">
         <v>274</v>
       </c>
-      <c r="B7" s="56">
+      <c r="B7" s="57">
         <f>COUNTIF('Feature List'!$G$5:$G$200,"Not Started")</f>
       </c>
-      <c r="C7" s="57">
+      <c r="C7" s="58">
         <f>IF(COUNTA('Feature List'!$G$5:$G$200)=0,0,COUNTIF('Feature List'!$G$5:$G$200,"Not Started")/COUNTA('Feature List'!$G$5:$G$200))</f>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="55" t="s">
-        <v>497</v>
-      </c>
-      <c r="B8" s="56">
+      <c r="A8" s="56" t="s">
+        <v>570</v>
+      </c>
+      <c r="B8" s="57">
         <f>COUNTIF('Feature List'!$G$5:$G$200,"Backlog")</f>
       </c>
-      <c r="C8" s="57">
+      <c r="C8" s="58">
         <f>IF(COUNTA('Feature List'!$G$5:$G$200)=0,0,COUNTIF('Feature List'!$G$5:$G$200,"Backlog")/COUNTA('Feature List'!$G$5:$G$200))</f>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="55" t="s">
-        <v>498</v>
-      </c>
-      <c r="B9" s="56">
+      <c r="A9" s="56" t="s">
+        <v>571</v>
+      </c>
+      <c r="B9" s="57">
         <f>COUNTIF('Feature List'!$G$5:$G$200,"Blocked")</f>
       </c>
-      <c r="C9" s="57">
+      <c r="C9" s="58">
         <f>IF(COUNTA('Feature List'!$G$5:$G$200)=0,0,COUNTIF('Feature List'!$G$5:$G$200,"Blocked")/COUNTA('Feature List'!$G$5:$G$200))</f>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="58" t="s">
-        <v>499</v>
-      </c>
-      <c r="B10" s="59">
+      <c r="A10" s="59" t="s">
+        <v>572</v>
+      </c>
+      <c r="B10" s="60">
         <f>COUNTA('Feature List'!$G$5:$G$200)</f>
       </c>
-      <c r="C10" s="60">
+      <c r="C10" s="61">
         <f>IF(COUNTA('Feature List'!$G$5:$G$200)=0,0,1)</f>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="53" t="s">
+      <c r="A12" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
+      <c r="B12" s="54"/>
+      <c r="C12" s="54"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="54" t="s">
+      <c r="A13" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="54" t="s">
-        <v>495</v>
-      </c>
-      <c r="C13" s="54" t="s">
-        <v>496</v>
+      <c r="B13" s="55" t="s">
+        <v>568</v>
+      </c>
+      <c r="C13" s="55" t="s">
+        <v>569</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="55" t="s">
+      <c r="A14" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="56">
+      <c r="B14" s="57">
         <f>COUNTIF('Feature List'!$I$5:$I$200,"Not Tested")</f>
       </c>
-      <c r="C14" s="57">
+      <c r="C14" s="58">
         <f>IF(COUNTA('Feature List'!$I$5:$I$200)=0,0,COUNTIF('Feature List'!$I$5:$I$200,"Not Tested")/COUNTA('Feature List'!$I$5:$I$200))</f>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="55" t="s">
+      <c r="A15" s="56" t="s">
         <v>314</v>
       </c>
-      <c r="B15" s="56">
+      <c r="B15" s="57">
         <f>COUNTIF('Feature List'!$I$5:$I$200,"In Progress")</f>
       </c>
-      <c r="C15" s="57">
+      <c r="C15" s="58">
         <f>IF(COUNTA('Feature List'!$I$5:$I$200)=0,0,COUNTIF('Feature List'!$I$5:$I$200,"In Progress")/COUNTA('Feature List'!$I$5:$I$200))</f>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="55" t="s">
+      <c r="A16" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="56">
+      <c r="B16" s="57">
         <f>COUNTIF('Feature List'!$I$5:$I$200,"Pass")</f>
       </c>
-      <c r="C16" s="57">
+      <c r="C16" s="58">
         <f>IF(COUNTA('Feature List'!$I$5:$I$200)=0,0,COUNTIF('Feature List'!$I$5:$I$200,"Pass")/COUNTA('Feature List'!$I$5:$I$200))</f>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="55" t="s">
-        <v>500</v>
-      </c>
-      <c r="B17" s="56">
+      <c r="A17" s="56" t="s">
+        <v>573</v>
+      </c>
+      <c r="B17" s="57">
         <f>COUNTIF('Feature List'!$I$5:$I$200,"Failed")</f>
       </c>
-      <c r="C17" s="57">
+      <c r="C17" s="58">
         <f>IF(COUNTA('Feature List'!$I$5:$I$200)=0,0,COUNTIF('Feature List'!$I$5:$I$200,"Failed")/COUNTA('Feature List'!$I$5:$I$200))</f>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="55" t="s">
-        <v>498</v>
-      </c>
-      <c r="B18" s="56">
+      <c r="A18" s="56" t="s">
+        <v>571</v>
+      </c>
+      <c r="B18" s="57">
         <f>COUNTIF('Feature List'!$I$5:$I$200,"Blocked")</f>
       </c>
-      <c r="C18" s="57">
+      <c r="C18" s="58">
         <f>IF(COUNTA('Feature List'!$I$5:$I$200)=0,0,COUNTIF('Feature List'!$I$5:$I$200,"Blocked")/COUNTA('Feature List'!$I$5:$I$200))</f>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="58" t="s">
-        <v>499</v>
-      </c>
-      <c r="B19" s="59">
+      <c r="A19" s="59" t="s">
+        <v>572</v>
+      </c>
+      <c r="B19" s="60">
         <f>COUNTA('Feature List'!$I$5:$I$200)</f>
       </c>
-      <c r="C19" s="60">
+      <c r="C19" s="61">
         <f>IF(COUNTA('Feature List'!$I$5:$I$200)=0,0,1)</f>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="53" t="s">
+      <c r="A21" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="53"/>
-      <c r="C21" s="53"/>
+      <c r="B21" s="54"/>
+      <c r="C21" s="54"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="54" t="s">
+      <c r="A22" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="B22" s="54" t="s">
-        <v>495</v>
-      </c>
-      <c r="C22" s="54" t="s">
-        <v>496</v>
+      <c r="B22" s="55" t="s">
+        <v>568</v>
+      </c>
+      <c r="C22" s="55" t="s">
+        <v>569</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="55" t="s">
+      <c r="A23" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="B23" s="56">
+      <c r="B23" s="57">
         <f>COUNTIF('Feature List'!$F$5:$F$200,"Existing")</f>
       </c>
-      <c r="C23" s="57">
+      <c r="C23" s="58">
         <f>IF(COUNTA('Feature List'!$F$5:$F$200)=0,0,COUNTIF('Feature List'!$F$5:$F$200,"Existing")/COUNTA('Feature List'!$F$5:$F$200))</f>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="55" t="s">
+      <c r="A24" s="56" t="s">
         <v>268</v>
       </c>
-      <c r="B24" s="56">
+      <c r="B24" s="57">
         <f>COUNTIF('Feature List'!$F$5:$F$200,"DevOps Backlog")</f>
       </c>
-      <c r="C24" s="57">
+      <c r="C24" s="58">
         <f>IF(COUNTA('Feature List'!$F$5:$F$200)=0,0,COUNTIF('Feature List'!$F$5:$F$200,"DevOps Backlog")/COUNTA('Feature List'!$F$5:$F$200))</f>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="55" t="s">
+      <c r="A25" s="56" t="s">
         <v>291</v>
       </c>
-      <c r="B25" s="56">
+      <c r="B25" s="57">
         <f>COUNTIF('Feature List'!$F$5:$F$200,"New Requirement")</f>
       </c>
-      <c r="C25" s="57">
+      <c r="C25" s="58">
         <f>IF(COUNTA('Feature List'!$F$5:$F$200)=0,0,COUNTIF('Feature List'!$F$5:$F$200,"New Requirement")/COUNTA('Feature List'!$F$5:$F$200))</f>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="58" t="s">
+      <c r="A26" s="59" t="s">
         <v>308</v>
       </c>
-      <c r="B26" s="59">
+      <c r="B26" s="60">
         <f>COUNTIF('Feature List'!$F$5:$F$200,"Nice to Have")</f>
       </c>
-      <c r="C26" s="60">
+      <c r="C26" s="61">
         <f>IF(COUNTA('Feature List'!$F$5:$F$200)=0,0,COUNTIF('Feature List'!$F$5:$F$200,"Nice to Have")/COUNTA('Feature List'!$F$5:$F$200))</f>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="58" t="s">
-        <v>499</v>
-      </c>
-      <c r="B27" s="59">
+      <c r="A27" s="59" t="s">
+        <v>572</v>
+      </c>
+      <c r="B27" s="60">
         <f>COUNTA('Feature List'!$F$5:$F$200)</f>
       </c>
-      <c r="C27" s="60">
+      <c r="C27" s="61">
         <f>IF(COUNTA('Feature List'!$F$5:$F$200)=0,0,1)</f>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="61" t="s">
-        <v>501</v>
-      </c>
-      <c r="B28" s="61"/>
-      <c r="C28" s="61"/>
+      <c r="A28" s="62" t="s">
+        <v>574</v>
+      </c>
+      <c r="B28" s="62"/>
+      <c r="C28" s="62"/>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="55" t="s">
-        <v>502</v>
-      </c>
-      <c r="B29" s="56">
+      <c r="A29" s="56" t="s">
+        <v>575</v>
+      </c>
+      <c r="B29" s="57">
         <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="55" t="s">
-        <v>503</v>
-      </c>
-      <c r="B30" s="56">
+      <c r="A30" s="56" t="s">
+        <v>576</v>
+      </c>
+      <c r="B30" s="57">
         <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="55" t="s">
-        <v>504</v>
-      </c>
-      <c r="B31" s="56">
+      <c r="A31" s="56" t="s">
+        <v>577</v>
+      </c>
+      <c r="B31" s="57">
         <v>4</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="55" t="s">
-        <v>505</v>
-      </c>
-      <c r="B32" s="56">
+      <c r="A32" s="56" t="s">
+        <v>578</v>
+      </c>
+      <c r="B32" s="57">
         <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="55" t="s">
-        <v>506</v>
-      </c>
-      <c r="B33" s="56">
+      <c r="A33" s="56" t="s">
+        <v>579</v>
+      </c>
+      <c r="B33" s="57">
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="55" t="s">
-        <v>507</v>
-      </c>
-      <c r="B34" s="56">
+      <c r="A34" s="56" t="s">
+        <v>580</v>
+      </c>
+      <c r="B34" s="57">
         <v>2</v>
       </c>
     </row>
@@ -7617,73 +8474,73 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="52" t="s">
-        <v>508</v>
-      </c>
-      <c r="B1" s="52"/>
+      <c r="A1" s="53" t="s">
+        <v>581</v>
+      </c>
+      <c r="B1" s="53"/>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="62" t="s">
-        <v>509</v>
-      </c>
-      <c r="B3" s="63" t="s">
-        <v>510</v>
+      <c r="A3" s="63" t="s">
+        <v>582</v>
+      </c>
+      <c r="B3" s="64" t="s">
+        <v>583</v>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="64" t="s">
+      <c r="A4" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="65" t="s">
-        <v>511</v>
+      <c r="B4" s="66" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="64" t="s">
+      <c r="A5" s="65" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="65" t="s">
-        <v>512</v>
+      <c r="B5" s="66" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="64" t="s">
+      <c r="A6" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="65" t="s">
-        <v>513</v>
+      <c r="B6" s="66" t="s">
+        <v>586</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="64" t="s">
+      <c r="A7" s="65" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="65" t="s">
-        <v>514</v>
+      <c r="B7" s="66" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="64" t="s">
+      <c r="A8" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="65" t="s">
-        <v>515</v>
+      <c r="B8" s="66" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="64" t="s">
+      <c r="A9" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="65" t="s">
-        <v>516</v>
+      <c r="B9" s="66" t="s">
+        <v>589</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="64" t="s">
-        <v>517</v>
-      </c>
-      <c r="B10" s="65" t="s">
-        <v>518</v>
+      <c r="A10" s="65" t="s">
+        <v>590</v>
+      </c>
+      <c r="B10" s="66" t="s">
+        <v>591</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(qa): add compare & As-Is Discovery rows; mark 3361/3362/3367 Pass
New rows added to Feature List sheet:
- #105 (3368) — Navigate to item from comparison diff card (comparison-links branch)
- #106 (3369) — As-Is Discovery page per process (client-as-is-discovery branch)
- #107 (3369) — As-Is Discovery data persisted per client version
- #108 (3369) — As-Is Discovery button in process panels

Stories 3361, 3362, 3367 updated from yellow/interim to green Pass
after confirmed testing.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MRI_Taxonomy_Feature_List_QA_v2.0.xlsx
+++ b/MRI_Taxonomy_Feature_List_QA_v2.0.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1531" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1571" uniqueCount="610">
   <si>
     <t>MRI ERP Implementation Taxonomy — Feature List &amp; QA Tracker</t>
   </si>
@@ -1219,7 +1219,7 @@
     <t>3361</t>
   </si>
   <si>
-    <t>Added 2026-10-01. DevOps User Story 3361. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+    <t>Added 2026-10-01. DevOps User Story 3361. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet. | Tested 2026-10-08 — Pass</t>
   </si>
   <si>
     <t>Propose a link that does not exist today</t>
@@ -1231,7 +1231,7 @@
     <t>3362</t>
   </si>
   <si>
-    <t>Added 2026-10-01. DevOps User Story 3362. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+    <t>Added 2026-10-01. DevOps User Story 3362. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet. | Tested 2026-10-08 — Pass</t>
   </si>
   <si>
     <t>Keep proposed links out of agreed-scope derivation</t>
@@ -1291,7 +1291,61 @@
     <t>3367</t>
   </si>
   <si>
-    <t>Added 2026-10-01. DevOps User Story 3367. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+    <t>Added 2026-10-01. DevOps User Story 3367. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet. | Tested 2026-10-08 — Pass</t>
+  </si>
+  <si>
+    <t>Navigate to an item from a comparison diff card</t>
+  </si>
+  <si>
+    <t>From each diff card in the comparison view, "Go to item" / "Open business process" / "Open MRI process" links jump directly to that changed item in the app. A "← Return to comparison" button re-opens the overlay at the same card. Navigation links are only shown when the item still exists in the current version.</t>
+  </si>
+  <si>
+    <t>src/components/compareView.js · setCompareNavigator() · src/main.js · compareView CSS</t>
+  </si>
+  <si>
+    <t>3368</t>
+  </si>
+  <si>
+    <t>Added 2026-10-08. comparison-links branch (commit 448b05b). Not yet merged to master.</t>
+  </si>
+  <si>
+    <t>Client Discovery</t>
+  </si>
+  <si>
+    <t>As-Is Discovery page per process</t>
+  </si>
+  <si>
+    <t>A full-page overlay accessible from any process panel (both Business and MRI System views) via an "As-Is Discovery" button. Captures: process narrative, roles &amp; responsibilities, frequency &amp; volume, tools &amp; workarounds, controls &amp; impact, evidence (source, date, participants, confidence), variations, and client target state. Criticality and discovery-status dropdowns update the badge bar instantly. "← Back to process" restores the panel.</t>
+  </si>
+  <si>
+    <t>src/components/discoveryPage.js · src/discoveryData.js · main.js · main.css</t>
+  </si>
+  <si>
+    <t>3369</t>
+  </si>
+  <si>
+    <t>Added 2026-10-08. client-as-is-discovery branch. Not yet merged to master.</t>
+  </si>
+  <si>
+    <t>As-Is Discovery data persisted per client version</t>
+  </si>
+  <si>
+    <t>Discovery data (all fields, criticality, status) is snapshotted when saving a version and restored when loading one. Data is blank when loading a version saved before this feature. Read-only in built-in baselines (Original and Discovery Baseline).</t>
+  </si>
+  <si>
+    <t>src/discoveryData.js · snapshotDiscovery() / restoreDiscovery() · main.js · versions.js</t>
+  </si>
+  <si>
+    <t>Added 2026-10-08. Part of story 3369 (client-as-is-discovery branch).</t>
+  </si>
+  <si>
+    <t>As-Is Discovery button in process panels</t>
+  </si>
+  <si>
+    <t>The "As-Is Discovery" button appears in the badge bar of both the MRI System panel and the Business Process panel. Clicking it opens the discovery overlay for that process, pre-loaded with any previously saved data.</t>
+  </si>
+  <si>
+    <t>src/components/panel.js · src/components/businessView.js · main.js (MutationObserver)</t>
   </si>
   <si>
     <t>DevOps Backlog ⇄ App Feature Comparison</t>
@@ -2623,7 +2677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K112"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -6123,10 +6177,10 @@
         <v>18</v>
       </c>
       <c r="H102" s="26" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="I102" s="26" t="s">
-        <v>309</v>
+        <v>30</v>
       </c>
       <c r="J102" s="26" t="s">
         <v>400</v>
@@ -6158,10 +6212,10 @@
         <v>18</v>
       </c>
       <c r="H103" s="26" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="I103" s="26" t="s">
-        <v>309</v>
+        <v>30</v>
       </c>
       <c r="J103" s="26" t="s">
         <v>404</v>
@@ -6333,16 +6387,156 @@
         <v>18</v>
       </c>
       <c r="H108" s="26" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="I108" s="26" t="s">
-        <v>309</v>
+        <v>30</v>
       </c>
       <c r="J108" s="26" t="s">
         <v>424</v>
       </c>
       <c r="K108" s="26" t="s">
         <v>425</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A109" s="25">
+        <v>105</v>
+      </c>
+      <c r="B109" s="25" t="s">
+        <v>186</v>
+      </c>
+      <c r="C109" s="25" t="s">
+        <v>426</v>
+      </c>
+      <c r="D109" s="25" t="s">
+        <v>427</v>
+      </c>
+      <c r="E109" s="25" t="s">
+        <v>428</v>
+      </c>
+      <c r="F109" s="25" t="s">
+        <v>268</v>
+      </c>
+      <c r="G109" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="H109" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="I109" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="J109" s="25" t="s">
+        <v>429</v>
+      </c>
+      <c r="K109" s="25" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A110" s="25">
+        <v>106</v>
+      </c>
+      <c r="B110" s="25" t="s">
+        <v>431</v>
+      </c>
+      <c r="C110" s="25" t="s">
+        <v>432</v>
+      </c>
+      <c r="D110" s="25" t="s">
+        <v>433</v>
+      </c>
+      <c r="E110" s="25" t="s">
+        <v>434</v>
+      </c>
+      <c r="F110" s="25" t="s">
+        <v>268</v>
+      </c>
+      <c r="G110" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="H110" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="I110" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="J110" s="25" t="s">
+        <v>435</v>
+      </c>
+      <c r="K110" s="25" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A111" s="25">
+        <v>107</v>
+      </c>
+      <c r="B111" s="25" t="s">
+        <v>431</v>
+      </c>
+      <c r="C111" s="25" t="s">
+        <v>437</v>
+      </c>
+      <c r="D111" s="25" t="s">
+        <v>438</v>
+      </c>
+      <c r="E111" s="25" t="s">
+        <v>439</v>
+      </c>
+      <c r="F111" s="25" t="s">
+        <v>268</v>
+      </c>
+      <c r="G111" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="H111" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="I111" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="J111" s="25" t="s">
+        <v>435</v>
+      </c>
+      <c r="K111" s="25" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A112" s="25">
+        <v>108</v>
+      </c>
+      <c r="B112" s="25" t="s">
+        <v>431</v>
+      </c>
+      <c r="C112" s="25" t="s">
+        <v>441</v>
+      </c>
+      <c r="D112" s="25" t="s">
+        <v>442</v>
+      </c>
+      <c r="E112" s="25" t="s">
+        <v>443</v>
+      </c>
+      <c r="F112" s="25" t="s">
+        <v>268</v>
+      </c>
+      <c r="G112" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="H112" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="I112" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="J112" s="25" t="s">
+        <v>435</v>
+      </c>
+      <c r="K112" s="25" t="s">
+        <v>440</v>
       </c>
     </row>
   </sheetData>
@@ -6399,7 +6593,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
-        <v>426</v>
+        <v>444</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -6412,7 +6606,7 @@
     </row>
     <row r="2" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="28" t="s">
-        <v>427</v>
+        <v>445</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -6425,7 +6619,7 @@
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
-        <v>428</v>
+        <v>446</v>
       </c>
       <c r="B3" s="29"/>
       <c r="C3" s="29"/>
@@ -6438,28 +6632,28 @@
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="30" t="s">
-        <v>429</v>
+        <v>447</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>430</v>
+        <v>448</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>431</v>
+        <v>449</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>432</v>
+        <v>450</v>
       </c>
       <c r="E4" s="30" t="s">
-        <v>433</v>
+        <v>451</v>
       </c>
       <c r="F4" s="30" t="s">
-        <v>434</v>
+        <v>452</v>
       </c>
       <c r="G4" s="30" t="s">
-        <v>435</v>
+        <v>453</v>
       </c>
       <c r="H4" s="30" t="s">
-        <v>436</v>
+        <v>454</v>
       </c>
       <c r="I4" s="30" t="s">
         <v>22</v>
@@ -6470,13 +6664,13 @@
         <v>21</v>
       </c>
       <c r="B5" s="32" t="s">
-        <v>437</v>
+        <v>455</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D5" s="34" t="s">
-        <v>439</v>
+        <v>457</v>
       </c>
       <c r="E5" s="33">
         <v>3</v>
@@ -6485,7 +6679,7 @@
         <v>14</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H5" s="32" t="s">
         <v>22</v>
@@ -6496,22 +6690,22 @@
         <v>40</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>441</v>
+        <v>459</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D6" s="39" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E6" s="38">
         <v>2</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>443</v>
+        <v>461</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H6" s="37" t="s">
         <v>22</v>
@@ -6519,25 +6713,25 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="31" t="s">
-        <v>444</v>
+        <v>462</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>445</v>
+        <v>463</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D7" s="34" t="s">
-        <v>439</v>
+        <v>457</v>
       </c>
       <c r="E7" s="33">
         <v>2</v>
       </c>
       <c r="F7" s="32" t="s">
-        <v>446</v>
+        <v>464</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H7" s="32" t="s">
         <v>22</v>
@@ -6548,13 +6742,13 @@
         <v>44</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>447</v>
+        <v>465</v>
       </c>
       <c r="C8" s="38" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D8" s="39" t="s">
-        <v>449</v>
+        <v>467</v>
       </c>
       <c r="E8" s="38">
         <v>3</v>
@@ -6563,7 +6757,7 @@
         <v>41</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H8" s="37" t="s">
         <v>22</v>
@@ -6574,22 +6768,22 @@
         <v>36</v>
       </c>
       <c r="B9" s="32" t="s">
-        <v>450</v>
+        <v>468</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D9" s="34" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E9" s="33">
         <v>3</v>
       </c>
       <c r="F9" s="32" t="s">
-        <v>451</v>
+        <v>469</v>
       </c>
       <c r="G9" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H9" s="32" t="s">
         <v>22</v>
@@ -6600,13 +6794,13 @@
         <v>97</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>452</v>
+        <v>470</v>
       </c>
       <c r="C10" s="38" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D10" s="39" t="s">
-        <v>453</v>
+        <v>471</v>
       </c>
       <c r="E10" s="38">
         <v>2</v>
@@ -6615,7 +6809,7 @@
         <v>94</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H10" s="37" t="s">
         <v>22</v>
@@ -6626,13 +6820,13 @@
         <v>74</v>
       </c>
       <c r="B11" s="32" t="s">
-        <v>454</v>
+        <v>472</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D11" s="34" t="s">
-        <v>453</v>
+        <v>471</v>
       </c>
       <c r="E11" s="33">
         <v>3</v>
@@ -6641,7 +6835,7 @@
         <v>71</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H11" s="32" t="s">
         <v>22</v>
@@ -6652,13 +6846,13 @@
         <v>78</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>455</v>
+        <v>473</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D12" s="39" t="s">
-        <v>439</v>
+        <v>457</v>
       </c>
       <c r="E12" s="38">
         <v>3</v>
@@ -6667,7 +6861,7 @@
         <v>75</v>
       </c>
       <c r="G12" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H12" s="37" t="s">
         <v>22</v>
@@ -6678,13 +6872,13 @@
         <v>81</v>
       </c>
       <c r="B13" s="32" t="s">
-        <v>456</v>
+        <v>474</v>
       </c>
       <c r="C13" s="33" t="s">
+        <v>475</v>
+      </c>
+      <c r="D13" s="34" t="s">
         <v>457</v>
-      </c>
-      <c r="D13" s="34" t="s">
-        <v>439</v>
       </c>
       <c r="E13" s="33">
         <v>2</v>
@@ -6693,7 +6887,7 @@
         <v>79</v>
       </c>
       <c r="G13" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H13" s="32" t="s">
         <v>22</v>
@@ -6704,13 +6898,13 @@
         <v>85</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>458</v>
+        <v>476</v>
       </c>
       <c r="C14" s="38" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D14" s="39" t="s">
-        <v>439</v>
+        <v>457</v>
       </c>
       <c r="E14" s="38">
         <v>2</v>
@@ -6719,7 +6913,7 @@
         <v>82</v>
       </c>
       <c r="G14" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H14" s="37" t="s">
         <v>22</v>
@@ -6730,13 +6924,13 @@
         <v>89</v>
       </c>
       <c r="B15" s="32" t="s">
-        <v>459</v>
+        <v>477</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D15" s="34" t="s">
-        <v>439</v>
+        <v>457</v>
       </c>
       <c r="E15" s="33">
         <v>2</v>
@@ -6745,7 +6939,7 @@
         <v>86</v>
       </c>
       <c r="G15" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H15" s="32" t="s">
         <v>22</v>
@@ -6756,22 +6950,22 @@
         <v>66</v>
       </c>
       <c r="B16" s="37" t="s">
+        <v>478</v>
+      </c>
+      <c r="C16" s="38" t="s">
+        <v>456</v>
+      </c>
+      <c r="D16" s="39" t="s">
         <v>460</v>
-      </c>
-      <c r="C16" s="38" t="s">
-        <v>438</v>
-      </c>
-      <c r="D16" s="39" t="s">
-        <v>442</v>
       </c>
       <c r="E16" s="38">
         <v>3</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>461</v>
+        <v>479</v>
       </c>
       <c r="G16" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H16" s="37" t="s">
         <v>22</v>
@@ -6782,22 +6976,22 @@
         <v>55</v>
       </c>
       <c r="B17" s="32" t="s">
-        <v>462</v>
+        <v>480</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D17" s="34" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E17" s="33">
         <v>3</v>
       </c>
       <c r="F17" s="32" t="s">
-        <v>463</v>
+        <v>481</v>
       </c>
       <c r="G17" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H17" s="32" t="s">
         <v>22</v>
@@ -6808,13 +7002,13 @@
         <v>174</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>464</v>
+        <v>482</v>
       </c>
       <c r="C18" s="38" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D18" s="40" t="s">
-        <v>465</v>
+        <v>483</v>
       </c>
       <c r="E18" s="38">
         <v>3</v>
@@ -6823,24 +7017,24 @@
         <v>175</v>
       </c>
       <c r="G18" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H18" s="37" t="s">
-        <v>466</v>
+        <v>484</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="31" t="s">
-        <v>467</v>
+        <v>485</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>468</v>
+        <v>486</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D19" s="41" t="s">
-        <v>465</v>
+        <v>483</v>
       </c>
       <c r="E19" s="33">
         <v>3</v>
@@ -6849,10 +7043,10 @@
         <v>118</v>
       </c>
       <c r="G19" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H19" s="32" t="s">
-        <v>466</v>
+        <v>484</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -6860,51 +7054,51 @@
         <v>185</v>
       </c>
       <c r="B20" s="37" t="s">
-        <v>469</v>
+        <v>487</v>
       </c>
       <c r="C20" s="38" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>465</v>
+        <v>483</v>
       </c>
       <c r="E20" s="38">
         <v>5</v>
       </c>
       <c r="F20" s="37" t="s">
-        <v>470</v>
+        <v>488</v>
       </c>
       <c r="G20" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H20" s="37" t="s">
-        <v>466</v>
+        <v>484</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="31" t="s">
-        <v>471</v>
+        <v>489</v>
       </c>
       <c r="B21" s="32" t="s">
-        <v>472</v>
+        <v>490</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D21" s="43" t="s">
-        <v>465</v>
+        <v>483</v>
       </c>
       <c r="E21" s="33">
         <v>3</v>
       </c>
       <c r="F21" s="32" t="s">
-        <v>473</v>
+        <v>491</v>
       </c>
       <c r="G21" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H21" s="32" t="s">
-        <v>466</v>
+        <v>484</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -6912,22 +7106,22 @@
         <v>104</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>474</v>
+        <v>492</v>
       </c>
       <c r="C22" s="38" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D22" s="39" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E22" s="38">
         <v>5</v>
       </c>
       <c r="F22" s="37" t="s">
-        <v>475</v>
+        <v>493</v>
       </c>
       <c r="G22" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H22" s="37" t="s">
         <v>22</v>
@@ -6938,13 +7132,13 @@
         <v>112</v>
       </c>
       <c r="B23" s="32" t="s">
-        <v>476</v>
+        <v>494</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D23" s="34" t="s">
-        <v>465</v>
+        <v>483</v>
       </c>
       <c r="E23" s="33">
         <v>3</v>
@@ -6953,7 +7147,7 @@
         <v>109</v>
       </c>
       <c r="G23" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H23" s="32" t="s">
         <v>22</v>
@@ -6964,13 +7158,13 @@
         <v>108</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>477</v>
+        <v>495</v>
       </c>
       <c r="C24" s="38" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D24" s="39" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E24" s="38">
         <v>3</v>
@@ -6979,7 +7173,7 @@
         <v>105</v>
       </c>
       <c r="G24" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H24" s="37" t="s">
         <v>22</v>
@@ -6987,16 +7181,16 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="31" t="s">
-        <v>478</v>
+        <v>496</v>
       </c>
       <c r="B25" s="32" t="s">
-        <v>479</v>
+        <v>497</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D25" s="34" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E25" s="33">
         <v>3</v>
@@ -7005,7 +7199,7 @@
         <v>158</v>
       </c>
       <c r="G25" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H25" s="32" t="s">
         <v>22</v>
@@ -7013,28 +7207,28 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="36" t="s">
-        <v>480</v>
+        <v>498</v>
       </c>
       <c r="B26" s="37" t="s">
-        <v>481</v>
+        <v>499</v>
       </c>
       <c r="C26" s="38" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D26" s="39" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="E26" s="38">
         <v>2</v>
       </c>
       <c r="F26" s="37" t="s">
-        <v>483</v>
+        <v>501</v>
       </c>
       <c r="G26" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H26" s="37" t="s">
-        <v>484</v>
+        <v>502</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -7042,13 +7236,13 @@
         <v>165</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>485</v>
+        <v>503</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D27" s="34" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E27" s="33">
         <v>3</v>
@@ -7057,7 +7251,7 @@
         <v>162</v>
       </c>
       <c r="G27" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H27" s="32" t="s">
         <v>22</v>
@@ -7068,13 +7262,13 @@
         <v>93</v>
       </c>
       <c r="B28" s="37" t="s">
-        <v>486</v>
+        <v>504</v>
       </c>
       <c r="C28" s="38" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D28" s="39" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E28" s="38">
         <v>3</v>
@@ -7083,7 +7277,7 @@
         <v>90</v>
       </c>
       <c r="G28" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H28" s="37" t="s">
         <v>22</v>
@@ -7091,25 +7285,25 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="31" t="s">
-        <v>487</v>
+        <v>505</v>
       </c>
       <c r="B29" s="32" t="s">
-        <v>488</v>
+        <v>506</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D29" s="34" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E29" s="33">
         <v>3</v>
       </c>
       <c r="F29" s="32" t="s">
-        <v>489</v>
+        <v>507</v>
       </c>
       <c r="G29" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H29" s="32" t="s">
         <v>22</v>
@@ -7120,13 +7314,13 @@
         <v>145</v>
       </c>
       <c r="B30" s="37" t="s">
-        <v>490</v>
+        <v>508</v>
       </c>
       <c r="C30" s="38" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D30" s="39" t="s">
-        <v>439</v>
+        <v>457</v>
       </c>
       <c r="E30" s="38">
         <v>3</v>
@@ -7135,7 +7329,7 @@
         <v>142</v>
       </c>
       <c r="G30" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H30" s="37" t="s">
         <v>22</v>
@@ -7146,13 +7340,13 @@
         <v>157</v>
       </c>
       <c r="B31" s="32" t="s">
-        <v>491</v>
+        <v>509</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D31" s="34" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="E31" s="33">
         <v>5</v>
@@ -7161,10 +7355,10 @@
         <v>154</v>
       </c>
       <c r="G31" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H31" s="32" t="s">
-        <v>492</v>
+        <v>510</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -7172,13 +7366,13 @@
         <v>149</v>
       </c>
       <c r="B32" s="37" t="s">
-        <v>493</v>
+        <v>511</v>
       </c>
       <c r="C32" s="38" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D32" s="39" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E32" s="38">
         <v>3</v>
@@ -7187,7 +7381,7 @@
         <v>146</v>
       </c>
       <c r="G32" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H32" s="37" t="s">
         <v>22</v>
@@ -7198,13 +7392,13 @@
         <v>153</v>
       </c>
       <c r="B33" s="32" t="s">
-        <v>494</v>
+        <v>512</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D33" s="34" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E33" s="33">
         <v>3</v>
@@ -7213,7 +7407,7 @@
         <v>150</v>
       </c>
       <c r="G33" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H33" s="32" t="s">
         <v>22</v>
@@ -7221,25 +7415,25 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="36" t="s">
-        <v>495</v>
+        <v>513</v>
       </c>
       <c r="B34" s="37" t="s">
-        <v>496</v>
+        <v>514</v>
       </c>
       <c r="C34" s="38" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D34" s="39" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E34" s="38">
         <v>5</v>
       </c>
       <c r="F34" s="37" t="s">
-        <v>497</v>
+        <v>515</v>
       </c>
       <c r="G34" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H34" s="37" t="s">
         <v>22</v>
@@ -7247,25 +7441,25 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="31" t="s">
-        <v>498</v>
+        <v>516</v>
       </c>
       <c r="B35" s="32" t="s">
-        <v>499</v>
+        <v>517</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D35" s="34" t="s">
-        <v>453</v>
+        <v>471</v>
       </c>
       <c r="E35" s="33">
         <v>5</v>
       </c>
       <c r="F35" s="32" t="s">
-        <v>500</v>
+        <v>518</v>
       </c>
       <c r="G35" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H35" s="32" t="s">
         <v>22</v>
@@ -7276,13 +7470,13 @@
         <v>262</v>
       </c>
       <c r="B36" s="37" t="s">
-        <v>501</v>
+        <v>519</v>
       </c>
       <c r="C36" s="38" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D36" s="39" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E36" s="38">
         <v>3</v>
@@ -7291,7 +7485,7 @@
         <v>259</v>
       </c>
       <c r="G36" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H36" s="37" t="s">
         <v>22</v>
@@ -7302,22 +7496,22 @@
         <v>190</v>
       </c>
       <c r="B37" s="32" t="s">
-        <v>502</v>
+        <v>520</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D37" s="34" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E37" s="33">
         <v>5</v>
       </c>
       <c r="F37" s="32" t="s">
-        <v>503</v>
+        <v>521</v>
       </c>
       <c r="G37" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H37" s="32" t="s">
         <v>22</v>
@@ -7328,13 +7522,13 @@
         <v>194</v>
       </c>
       <c r="B38" s="37" t="s">
-        <v>504</v>
+        <v>522</v>
       </c>
       <c r="C38" s="38" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="D38" s="39" t="s">
-        <v>465</v>
+        <v>483</v>
       </c>
       <c r="E38" s="38">
         <v>3</v>
@@ -7343,7 +7537,7 @@
         <v>191</v>
       </c>
       <c r="G38" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H38" s="37" t="s">
         <v>22</v>
@@ -7354,13 +7548,13 @@
         <v>211</v>
       </c>
       <c r="B39" s="32" t="s">
-        <v>505</v>
+        <v>523</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D39" s="34" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E39" s="33">
         <v>3</v>
@@ -7369,7 +7563,7 @@
         <v>208</v>
       </c>
       <c r="G39" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H39" s="32" t="s">
         <v>22</v>
@@ -7380,22 +7574,22 @@
         <v>215</v>
       </c>
       <c r="B40" s="37" t="s">
-        <v>506</v>
+        <v>524</v>
       </c>
       <c r="C40" s="38" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D40" s="39" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E40" s="38">
         <v>2</v>
       </c>
       <c r="F40" s="37" t="s">
-        <v>507</v>
+        <v>525</v>
       </c>
       <c r="G40" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H40" s="37" t="s">
         <v>22</v>
@@ -7406,25 +7600,25 @@
         <v>223</v>
       </c>
       <c r="B41" s="32" t="s">
-        <v>508</v>
+        <v>526</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D41" s="34" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E41" s="33">
         <v>3</v>
       </c>
       <c r="F41" s="32" t="s">
-        <v>509</v>
+        <v>527</v>
       </c>
       <c r="G41" s="35" t="s">
-        <v>510</v>
+        <v>528</v>
       </c>
       <c r="H41" s="32" t="s">
-        <v>511</v>
+        <v>529</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -7432,22 +7626,22 @@
         <v>238</v>
       </c>
       <c r="B42" s="37" t="s">
-        <v>512</v>
+        <v>530</v>
       </c>
       <c r="C42" s="38" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D42" s="39" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E42" s="38">
         <v>5</v>
       </c>
       <c r="F42" s="37" t="s">
-        <v>513</v>
+        <v>531</v>
       </c>
       <c r="G42" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H42" s="37" t="s">
         <v>22</v>
@@ -7458,13 +7652,13 @@
         <v>242</v>
       </c>
       <c r="B43" s="32" t="s">
-        <v>514</v>
+        <v>532</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="D43" s="34" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E43" s="33">
         <v>3</v>
@@ -7473,7 +7667,7 @@
         <v>239</v>
       </c>
       <c r="G43" s="35" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="H43" s="32" t="s">
         <v>22</v>
@@ -7481,7 +7675,7 @@
     </row>
     <row r="45" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="44" t="s">
-        <v>515</v>
+        <v>533</v>
       </c>
       <c r="B45" s="44"/>
       <c r="C45" s="44"/>
@@ -7494,25 +7688,25 @@
     </row>
     <row r="46" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="30" t="s">
-        <v>429</v>
+        <v>447</v>
       </c>
       <c r="B46" s="30" t="s">
-        <v>430</v>
+        <v>448</v>
       </c>
       <c r="C46" s="30" t="s">
-        <v>431</v>
+        <v>449</v>
       </c>
       <c r="D46" s="30" t="s">
-        <v>432</v>
+        <v>450</v>
       </c>
       <c r="E46" s="30" t="s">
-        <v>433</v>
+        <v>451</v>
       </c>
       <c r="F46" s="30" t="s">
-        <v>435</v>
+        <v>453</v>
       </c>
       <c r="G46" s="30" t="s">
-        <v>516</v>
+        <v>534</v>
       </c>
       <c r="H46" s="30" t="s">
         <v>22</v>
@@ -7529,19 +7723,19 @@
         <v>265</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D47" s="32" t="s">
-        <v>465</v>
+        <v>483</v>
       </c>
       <c r="E47" s="33">
         <v>2</v>
       </c>
       <c r="F47" s="45" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="G47" s="32" t="s">
-        <v>517</v>
+        <v>535</v>
       </c>
       <c r="H47" s="32"/>
       <c r="I47" s="32"/>
@@ -7551,22 +7745,22 @@
         <v>275</v>
       </c>
       <c r="B48" s="32" t="s">
-        <v>518</v>
+        <v>536</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D48" s="32" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="E48" s="33">
         <v>2</v>
       </c>
       <c r="F48" s="46" t="s">
-        <v>519</v>
+        <v>537</v>
       </c>
       <c r="G48" s="32" t="s">
-        <v>520</v>
+        <v>538</v>
       </c>
       <c r="H48" s="32"/>
       <c r="I48" s="32"/>
@@ -7579,19 +7773,19 @@
         <v>278</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>521</v>
+        <v>539</v>
       </c>
       <c r="D49" s="32" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="E49" s="33">
         <v>8</v>
       </c>
       <c r="F49" s="46" t="s">
-        <v>519</v>
+        <v>537</v>
       </c>
       <c r="G49" s="32" t="s">
-        <v>522</v>
+        <v>540</v>
       </c>
       <c r="H49" s="32"/>
       <c r="I49" s="32"/>
@@ -7601,29 +7795,29 @@
         <v>286</v>
       </c>
       <c r="B50" s="32" t="s">
-        <v>523</v>
+        <v>541</v>
       </c>
       <c r="C50" s="33" t="s">
-        <v>521</v>
+        <v>539</v>
       </c>
       <c r="D50" s="32" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="E50" s="33">
         <v>5</v>
       </c>
       <c r="F50" s="46" t="s">
-        <v>519</v>
+        <v>537</v>
       </c>
       <c r="G50" s="32" t="s">
-        <v>524</v>
+        <v>542</v>
       </c>
       <c r="H50" s="32"/>
       <c r="I50" s="32"/>
     </row>
     <row r="52" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="47" t="s">
-        <v>525</v>
+        <v>543</v>
       </c>
       <c r="B52" s="47"/>
       <c r="C52" s="47"/>
@@ -7645,7 +7839,7 @@
         <v>6</v>
       </c>
       <c r="D53" s="30" t="s">
-        <v>526</v>
+        <v>544</v>
       </c>
       <c r="E53" s="30" t="s">
         <v>22</v>
@@ -7674,7 +7868,7 @@
         <v>25</v>
       </c>
       <c r="D54" s="32" t="s">
-        <v>527</v>
+        <v>545</v>
       </c>
       <c r="E54" s="32"/>
       <c r="F54" s="32"/>
@@ -7693,7 +7887,7 @@
         <v>47</v>
       </c>
       <c r="D55" s="32" t="s">
-        <v>528</v>
+        <v>546</v>
       </c>
       <c r="E55" s="32"/>
       <c r="F55" s="32"/>
@@ -7712,7 +7906,7 @@
         <v>140</v>
       </c>
       <c r="D56" s="32" t="s">
-        <v>529</v>
+        <v>547</v>
       </c>
       <c r="E56" s="32"/>
       <c r="F56" s="32"/>
@@ -7731,7 +7925,7 @@
         <v>197</v>
       </c>
       <c r="D57" s="32" t="s">
-        <v>530</v>
+        <v>548</v>
       </c>
       <c r="E57" s="32"/>
       <c r="F57" s="32"/>
@@ -7750,7 +7944,7 @@
         <v>206</v>
       </c>
       <c r="D58" s="32" t="s">
-        <v>531</v>
+        <v>549</v>
       </c>
       <c r="E58" s="32"/>
       <c r="F58" s="32"/>
@@ -7760,7 +7954,7 @@
     </row>
     <row r="60" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="50" t="s">
-        <v>532</v>
+        <v>550</v>
       </c>
       <c r="B60" s="50"/>
       <c r="C60" s="50"/>
@@ -7782,13 +7976,13 @@
         <v>5</v>
       </c>
       <c r="D61" s="30" t="s">
-        <v>533</v>
+        <v>551</v>
       </c>
       <c r="E61" s="30" t="s">
         <v>8</v>
       </c>
       <c r="F61" s="30" t="s">
-        <v>534</v>
+        <v>552</v>
       </c>
       <c r="G61" s="30" t="s">
         <v>22</v>
@@ -7808,16 +8002,16 @@
         <v>67</v>
       </c>
       <c r="C62" s="32" t="s">
-        <v>535</v>
+        <v>553</v>
       </c>
       <c r="D62" s="32" t="s">
-        <v>536</v>
+        <v>554</v>
       </c>
       <c r="E62" s="51" t="s">
-        <v>465</v>
+        <v>483</v>
       </c>
       <c r="F62" s="52" t="s">
-        <v>537</v>
+        <v>555</v>
       </c>
       <c r="G62" s="52"/>
       <c r="H62" s="52"/>
@@ -7831,16 +8025,16 @@
         <v>67</v>
       </c>
       <c r="C63" s="32" t="s">
-        <v>538</v>
+        <v>556</v>
       </c>
       <c r="D63" s="32" t="s">
-        <v>539</v>
+        <v>557</v>
       </c>
       <c r="E63" s="51" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="F63" s="52" t="s">
-        <v>540</v>
+        <v>558</v>
       </c>
       <c r="G63" s="52"/>
       <c r="H63" s="52"/>
@@ -7854,16 +8048,16 @@
         <v>141</v>
       </c>
       <c r="C64" s="32" t="s">
-        <v>541</v>
+        <v>559</v>
       </c>
       <c r="D64" s="32" t="s">
-        <v>542</v>
+        <v>560</v>
       </c>
       <c r="E64" s="51" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="F64" s="52" t="s">
-        <v>543</v>
+        <v>561</v>
       </c>
       <c r="G64" s="52"/>
       <c r="H64" s="52"/>
@@ -7877,16 +8071,16 @@
         <v>299</v>
       </c>
       <c r="C65" s="32" t="s">
-        <v>544</v>
+        <v>562</v>
       </c>
       <c r="D65" s="32" t="s">
-        <v>545</v>
+        <v>563</v>
       </c>
       <c r="E65" s="51" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="F65" s="52" t="s">
-        <v>546</v>
+        <v>564</v>
       </c>
       <c r="G65" s="52"/>
       <c r="H65" s="52"/>
@@ -7900,16 +8094,16 @@
         <v>186</v>
       </c>
       <c r="C66" s="32" t="s">
-        <v>547</v>
+        <v>565</v>
       </c>
       <c r="D66" s="32" t="s">
-        <v>548</v>
+        <v>566</v>
       </c>
       <c r="E66" s="51" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="F66" s="52" t="s">
-        <v>549</v>
+        <v>567</v>
       </c>
       <c r="G66" s="52"/>
       <c r="H66" s="52"/>
@@ -7917,7 +8111,7 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="44" t="s">
-        <v>550</v>
+        <v>568</v>
       </c>
       <c r="B68" s="44"/>
       <c r="C68" s="44"/>
@@ -7928,163 +8122,163 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="30" t="s">
-        <v>429</v>
+        <v>447</v>
       </c>
       <c r="B69" s="30" t="s">
-        <v>430</v>
+        <v>448</v>
       </c>
       <c r="C69" s="30" t="s">
-        <v>431</v>
+        <v>449</v>
       </c>
       <c r="D69" s="30" t="s">
-        <v>432</v>
+        <v>450</v>
       </c>
       <c r="E69" s="30" t="s">
-        <v>433</v>
+        <v>451</v>
       </c>
       <c r="F69" s="30" t="s">
-        <v>435</v>
+        <v>453</v>
       </c>
       <c r="G69" s="30" t="s">
-        <v>516</v>
+        <v>534</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="31" t="s">
-        <v>551</v>
+        <v>569</v>
       </c>
       <c r="B70" s="32" t="s">
         <v>306</v>
       </c>
       <c r="C70" s="33" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D70" s="32" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="E70" s="33">
         <v>8</v>
       </c>
       <c r="F70" s="45" t="s">
-        <v>519</v>
+        <v>537</v>
       </c>
       <c r="G70" s="32" t="s">
-        <v>552</v>
+        <v>570</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="31" t="s">
-        <v>553</v>
+        <v>571</v>
       </c>
       <c r="B71" s="32" t="s">
         <v>311</v>
       </c>
       <c r="C71" s="33" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D71" s="32" t="s">
-        <v>554</v>
+        <v>572</v>
       </c>
       <c r="E71" s="33">
         <v>13</v>
       </c>
       <c r="F71" s="46" t="s">
-        <v>519</v>
+        <v>537</v>
       </c>
       <c r="G71" s="32" t="s">
-        <v>555</v>
+        <v>573</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="31" t="s">
-        <v>556</v>
+        <v>574</v>
       </c>
       <c r="B72" s="32" t="s">
         <v>316</v>
       </c>
       <c r="C72" s="33" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D72" s="32" t="s">
-        <v>465</v>
+        <v>483</v>
       </c>
       <c r="E72" s="33">
         <v>3</v>
       </c>
       <c r="F72" s="45" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="G72" s="32" t="s">
-        <v>557</v>
+        <v>575</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="31" t="s">
-        <v>558</v>
+        <v>576</v>
       </c>
       <c r="B73" s="32" t="s">
         <v>320</v>
       </c>
       <c r="C73" s="33" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D73" s="32" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="E73" s="33">
         <v>8</v>
       </c>
       <c r="F73" s="46" t="s">
-        <v>510</v>
+        <v>528</v>
       </c>
       <c r="G73" s="32" t="s">
-        <v>559</v>
+        <v>577</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="31" t="s">
-        <v>560</v>
+        <v>578</v>
       </c>
       <c r="B74" s="32" t="s">
         <v>324</v>
       </c>
       <c r="C74" s="33" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D74" s="32" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="E74" s="33">
         <v>8</v>
       </c>
       <c r="F74" s="45" t="s">
-        <v>519</v>
+        <v>537</v>
       </c>
       <c r="G74" s="32" t="s">
-        <v>561</v>
+        <v>579</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="31" t="s">
-        <v>562</v>
+        <v>580</v>
       </c>
       <c r="B75" s="32" t="s">
         <v>327</v>
       </c>
       <c r="C75" s="33" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D75" s="32" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="E75" s="33">
         <v>8</v>
       </c>
       <c r="F75" s="46" t="s">
-        <v>519</v>
+        <v>537</v>
       </c>
       <c r="G75" s="32" t="s">
-        <v>563</v>
+        <v>581</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
@@ -8095,19 +8289,19 @@
         <v>330</v>
       </c>
       <c r="C76" s="33" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="D76" s="32" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="E76" s="33" t="s">
-        <v>564</v>
+        <v>582</v>
       </c>
       <c r="F76" s="45" t="s">
-        <v>519</v>
+        <v>537</v>
       </c>
       <c r="G76" s="32" t="s">
-        <v>565</v>
+        <v>583</v>
       </c>
     </row>
   </sheetData>
@@ -8150,14 +8344,14 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="53" t="s">
-        <v>566</v>
+        <v>584</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
     </row>
     <row r="3" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="54" t="s">
-        <v>567</v>
+        <v>585</v>
       </c>
       <c r="B3" s="54"/>
       <c r="C3" s="54"/>
@@ -8167,10 +8361,10 @@
         <v>8</v>
       </c>
       <c r="B4" s="55" t="s">
-        <v>568</v>
+        <v>586</v>
       </c>
       <c r="C4" s="55" t="s">
-        <v>569</v>
+        <v>587</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -8208,7 +8402,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="56" t="s">
-        <v>570</v>
+        <v>588</v>
       </c>
       <c r="B8" s="57">
         <f>COUNTIF('Feature List'!$G$5:$G$200,"Backlog")</f>
@@ -8219,7 +8413,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="56" t="s">
-        <v>571</v>
+        <v>589</v>
       </c>
       <c r="B9" s="57">
         <f>COUNTIF('Feature List'!$G$5:$G$200,"Blocked")</f>
@@ -8230,7 +8424,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="59" t="s">
-        <v>572</v>
+        <v>590</v>
       </c>
       <c r="B10" s="60">
         <f>COUNTA('Feature List'!$G$5:$G$200)</f>
@@ -8251,10 +8445,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="55" t="s">
-        <v>568</v>
+        <v>586</v>
       </c>
       <c r="C13" s="55" t="s">
-        <v>569</v>
+        <v>587</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -8292,7 +8486,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="56" t="s">
-        <v>573</v>
+        <v>591</v>
       </c>
       <c r="B17" s="57">
         <f>COUNTIF('Feature List'!$I$5:$I$200,"Failed")</f>
@@ -8303,7 +8497,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="56" t="s">
-        <v>571</v>
+        <v>589</v>
       </c>
       <c r="B18" s="57">
         <f>COUNTIF('Feature List'!$I$5:$I$200,"Blocked")</f>
@@ -8314,7 +8508,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="59" t="s">
-        <v>572</v>
+        <v>590</v>
       </c>
       <c r="B19" s="60">
         <f>COUNTA('Feature List'!$I$5:$I$200)</f>
@@ -8335,10 +8529,10 @@
         <v>7</v>
       </c>
       <c r="B22" s="55" t="s">
-        <v>568</v>
+        <v>586</v>
       </c>
       <c r="C22" s="55" t="s">
-        <v>569</v>
+        <v>587</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -8387,7 +8581,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="59" t="s">
-        <v>572</v>
+        <v>590</v>
       </c>
       <c r="B27" s="60">
         <f>COUNTA('Feature List'!$F$5:$F$200)</f>
@@ -8398,14 +8592,14 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="62" t="s">
-        <v>574</v>
+        <v>592</v>
       </c>
       <c r="B28" s="62"/>
       <c r="C28" s="62"/>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="56" t="s">
-        <v>575</v>
+        <v>593</v>
       </c>
       <c r="B29" s="57">
         <v>60</v>
@@ -8413,7 +8607,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="56" t="s">
-        <v>576</v>
+        <v>594</v>
       </c>
       <c r="B30" s="57">
         <v>60</v>
@@ -8421,7 +8615,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="56" t="s">
-        <v>577</v>
+        <v>595</v>
       </c>
       <c r="B31" s="57">
         <v>4</v>
@@ -8429,7 +8623,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="56" t="s">
-        <v>578</v>
+        <v>596</v>
       </c>
       <c r="B32" s="57">
         <v>4</v>
@@ -8437,7 +8631,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="56" t="s">
-        <v>579</v>
+        <v>597</v>
       </c>
       <c r="B33" s="57">
         <v>0</v>
@@ -8445,7 +8639,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="56" t="s">
-        <v>580</v>
+        <v>598</v>
       </c>
       <c r="B34" s="57">
         <v>2</v>
@@ -8475,16 +8669,16 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="53" t="s">
-        <v>581</v>
+        <v>599</v>
       </c>
       <c r="B1" s="53"/>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="63" t="s">
-        <v>582</v>
+        <v>600</v>
       </c>
       <c r="B3" s="64" t="s">
-        <v>583</v>
+        <v>601</v>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -8492,7 +8686,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="66" t="s">
-        <v>584</v>
+        <v>602</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -8500,7 +8694,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="66" t="s">
-        <v>585</v>
+        <v>603</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -8508,7 +8702,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="66" t="s">
-        <v>586</v>
+        <v>604</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -8516,7 +8710,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="66" t="s">
-        <v>587</v>
+        <v>605</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -8524,7 +8718,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="66" t="s">
-        <v>588</v>
+        <v>606</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -8532,15 +8726,15 @@
         <v>12</v>
       </c>
       <c r="B9" s="66" t="s">
-        <v>589</v>
+        <v>607</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="65" t="s">
-        <v>590</v>
+        <v>608</v>
       </c>
       <c r="B10" s="66" t="s">
-        <v>591</v>
+        <v>609</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(qa): mark feature rows 96-101 (3359/3360/3363/3364) Tested/Pass
Stories 3361 and 3362 were already Pass; skipped.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MRI_Taxonomy_Feature_List_QA_v2.0.xlsx
+++ b/MRI_Taxonomy_Feature_List_QA_v2.0.xlsx
@@ -1195,7 +1195,7 @@
     <t>3359</t>
   </si>
   <si>
-    <t>Added 2026-10-01. DevOps Feature 3359. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+    <t>Added 2026-10-01. DevOps Feature 3359. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet. | Tested 2026-10-08: Pass</t>
   </si>
   <si>
     <t>Imply a proposal across links in both directions</t>
@@ -1207,7 +1207,7 @@
     <t>3360</t>
   </si>
   <si>
-    <t>Added 2026-10-01. DevOps User Story 3360. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+    <t>Added 2026-10-01. DevOps User Story 3360. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet. | Tested 2026-10-08: Pass</t>
   </si>
   <si>
     <t>Prevent proposal propagation from cascading</t>
@@ -1243,7 +1243,7 @@
     <t>3363</t>
   </si>
   <si>
-    <t>Added 2026-10-01. DevOps User Story 3363. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+    <t>Added 2026-10-01. DevOps User Story 3363. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet. | Tested 2026-10-08: Pass</t>
   </si>
   <si>
     <t>Value-Add Proposals Document</t>
@@ -1255,7 +1255,7 @@
     <t>3364</t>
   </si>
   <si>
-    <t>Added 2026-10-01. DevOps Feature 3364. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet.</t>
+    <t>Added 2026-10-01. DevOps Feature 3364. Implementation confirmed present by code inspection; core flow (propose a card, filter by Proposed Scope) smoke-tested in browser — no formal QA test pass run yet. | Tested 2026-10-08: Pass</t>
   </si>
   <si>
     <t>Exclude proposals from generated documents by default</t>
@@ -6107,10 +6107,10 @@
         <v>18</v>
       </c>
       <c r="H100" s="26" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="I100" s="26" t="s">
-        <v>309</v>
+        <v>30</v>
       </c>
       <c r="J100" s="26" t="s">
         <v>392</v>
@@ -6142,10 +6142,10 @@
         <v>18</v>
       </c>
       <c r="H101" s="26" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="I101" s="26" t="s">
-        <v>309</v>
+        <v>30</v>
       </c>
       <c r="J101" s="26" t="s">
         <v>396</v>
@@ -6247,10 +6247,10 @@
         <v>18</v>
       </c>
       <c r="H104" s="26" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="I104" s="26" t="s">
-        <v>309</v>
+        <v>30</v>
       </c>
       <c r="J104" s="26" t="s">
         <v>408</v>
@@ -6282,10 +6282,10 @@
         <v>18</v>
       </c>
       <c r="H105" s="26" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="I105" s="26" t="s">
-        <v>309</v>
+        <v>30</v>
       </c>
       <c r="J105" s="26" t="s">
         <v>412</v>

</xml_diff>